<commit_message>
automating more analysis in table 1
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
   <si>
     <t xml:space="preserve">signature id</t>
   </si>
@@ -80,532 +80,511 @@
     <t xml:space="preserve">Biliary::DRUP01010095T</t>
   </si>
   <si>
+    <t xml:space="preserve">InD1*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::SP21400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel1c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver::SP49229</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bone.SoftTissue::CPCT02020428T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esophagus::CPCT02010569T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::SP96118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lymphoid::CPCT02120032T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lung::SP58101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other::CPCT02020815T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNS::CPCT02100089T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD4a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel5a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kidney::SP39298</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel5b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver::SP112290</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ovary::SP62616</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uterus::SP94741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID7**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breast::SP116365</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pancreas::SP102617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD9b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other::SP109957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID10**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pancreas::SP77956</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prostate::SP112985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skin::SP124439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD13*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::CPCT02040258T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WES::TCGA-EW-A2FV-01A-11D-A17D-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WES::TCGA-13-0889-01A-01W-0420-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other::CPCT02250003T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head::CPCT02070053T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bone.SoftTissue::CPCT02010408T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skin::CPCT02340081T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skin::CPCT02060041T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kidney::SP102957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_A_alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other::CPCT02330041T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD9a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_A_beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breast::SP2293</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD9a*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver::CPCT02020413T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breast::CPCT02010772T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::CPCT02340014T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD12*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uterus::DRUP01340014T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Head::DRUP01030028T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other::DRUP01030015T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bone.SoftTissue::CPCT02010648T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNS::SP107439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::DRUP01230004T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_J**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_K_alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prostate::SP112817</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_K_beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon::SP17905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pancreas::SP70106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prostate::SP112777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stomach::CPCT02030347T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_N**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CNS::CPCT02100101T</t>
+  </si>
+  <si>
     <t xml:space="preserve">InD1</t>
   </si>
   <si>
-    <t xml:space="preserve">C_ID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel1b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::SP21400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel1c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liver::SP49229</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel1d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bone.SoftTissue::CPCT02020428T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esophagus::CPCT02010569T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD2b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::SP96118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lymphoid::CPCT02120032T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lung::SP58101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel3b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other::CPCT02020815T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD3b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CNS::CPCT02100089T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD4a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel5a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kidney::SP39298</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel5b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liver::SP112290</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ovary::SP62616</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uterus::SP94741</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID7*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breast::SP116365</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pancreas::SP102617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD9b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other::SP109957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID10*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pancreas::SP77956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID11a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prostate::SP112985</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skin::SP124439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::CPCT02040258T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WES::TCGA-EW-A2FV-01A-11D-A17D-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WES::TCGA-13-0889-01A-01W-0420-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other::CPCT02250003T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Head::CPCT02070053T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bone.SoftTissue::CPCT02010408T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skin::CPCT02340081T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skin::CPCT02060041T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kidney::SP102957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_A_alpha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other::CPCT02330041T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD9a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_A_beta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breast::SP2293</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liver::CPCT02020413T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breast::CPCT02010772T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::CPCT02340014T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uterus::DRUP01340014T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Head::DRUP01030028T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other::DRUP01030015T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID11b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bone.SoftTissue::CPCT02010648T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CNS::SP107439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::DRUP01230004T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_J*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_K_alpha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prostate::SP112817</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jinID26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_K_beta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colon::SP17905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pancreas::SP70106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prostate::SP112777</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stomach::CPCT02030347T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_N*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CNS::CPCT02100101T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_O*</t>
+    <t xml:space="preserve">ID_O**</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel_P</t>
@@ -620,17 +599,21 @@
     <t xml:space="preserve">ID_P</t>
   </si>
   <si>
-    <t xml:space="preserve">* indicates that in the supporting tumor's spectrum, insertions of a single T in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
+    <t xml:space="preserve">* This is the signature with the best match to the given signature_id.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">** indicates that in the supporting tumor's spectrum, insertions of a single T in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -647,6 +630,11 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFB0B0B0"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -670,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -679,6 +667,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -981,14 +975,14 @@
     <col min="2" max="2" width="8.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="35.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="7.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="8.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="8.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="8.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="9.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="10.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="8.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="6.71" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="8.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="10.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="8.71" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="7.71" hidden="0" customWidth="1"/>
@@ -1083,22 +1077,22 @@
       <c r="G2" s="3" t="n">
         <v>0.9596639524824</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="7" t="n">
         <v>0.998418245662758</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="5" t="n">
+      <c r="L2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="7" t="n">
         <v>0.998577618888331</v>
       </c>
       <c r="N2" s="3" t="n">
@@ -1125,19 +1119,19 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.995824348751852</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0.987184801324652</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.961293866458291</v>
@@ -1145,22 +1139,22 @@
       <c r="G3" s="3" t="n">
         <v>0.971169546248927</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="7" t="n">
         <v>0.961390178570747</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K3" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
-      <c r="L3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M3" s="5" t="n">
+      <c r="L3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="7" t="n">
         <v>0.998577618888331</v>
       </c>
       <c r="N3" s="3" t="n">
@@ -1187,19 +1181,19 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.961311961936925</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0.923032940882415</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.93647989440547</v>
@@ -1207,22 +1201,22 @@
       <c r="G4" s="3" t="n">
         <v>0.929054257037847</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="7" t="n">
         <v>0.998493112709776</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
-      <c r="L4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M4" s="5" t="n">
+      <c r="L4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="7" t="n">
         <v>0.998577618888331</v>
       </c>
       <c r="N4" s="3" t="n">
@@ -1249,13 +1243,13 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.997816677302374</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0.99675737544784</v>
@@ -1265,22 +1259,22 @@
       <c r="G5" s="3" t="n">
         <v>0.994594220752138</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="7" t="n">
         <v>0.99606877275794</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
-      <c r="L5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" s="5" t="n">
+      <c r="L5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="7" t="n">
         <v>0.998577618888331</v>
       </c>
       <c r="N5" s="3" t="n">
@@ -1307,19 +1301,19 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.980501734047094</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.990263031835387</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0.905687533553426</v>
@@ -1327,22 +1321,22 @@
       <c r="G6" s="3" t="n">
         <v>0.967949920301316</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.896138732515832</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>0.896138732515832</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
-      <c r="L6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M6" s="5" t="n">
+      <c r="L6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="7" t="n">
         <v>0.998910219006335</v>
       </c>
       <c r="N6" s="3" t="n">
@@ -1369,13 +1363,13 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.985087090067255</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0.933667457882778</v>
@@ -1385,22 +1379,22 @@
       <c r="G7" s="3" t="n">
         <v>0.931852177125591</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>0.955583423187771</v>
+      </c>
+      <c r="J7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>0.955583423187771</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
-      <c r="L7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" s="5" t="n">
+      <c r="L7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="M7" s="7" t="n">
         <v>0.998910219006335</v>
       </c>
       <c r="N7" s="3" t="n">
@@ -1427,13 +1421,13 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0.983098547202523</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0.979438082042213</v>
@@ -1443,22 +1437,22 @@
       <c r="G8" s="3" t="n">
         <v>0.999362829413946</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0.982691257770152</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>0.982691257770152</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
-      <c r="L8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="M8" s="5" t="n">
+      <c r="L8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" s="7" t="n">
         <v>0.998910219006335</v>
       </c>
       <c r="N8" s="3" t="n">
@@ -1485,19 +1479,19 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.995407107687552</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0.953117492152762</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0.913569151804241</v>
@@ -1505,22 +1499,22 @@
       <c r="G9" s="3" t="n">
         <v>0.893003527564203</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" s="5" t="n">
+      <c r="H9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="7" t="n">
         <v>0.90592938388244</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K9" s="5" t="n">
+      <c r="J9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K9" s="7" t="n">
         <v>0.992673228868062</v>
       </c>
-      <c r="L9" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="M9" s="5" t="n">
+      <c r="L9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M9" s="7" t="n">
         <v>0.952591756729311</v>
       </c>
       <c r="N9" s="3" t="n">
@@ -1547,19 +1541,19 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.99886526497977</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.992284649786581</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0.953522795429812</v>
@@ -1567,22 +1561,22 @@
       <c r="G10" s="3" t="n">
         <v>0.990426082637624</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" s="5" t="n">
+      <c r="H10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" s="7" t="n">
         <v>0.988504232948747</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K10" s="5" t="n">
+      <c r="J10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K10" s="7" t="n">
         <v>0.992673228868062</v>
       </c>
-      <c r="L10" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="M10" s="5" t="n">
+      <c r="L10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M10" s="7" t="n">
         <v>0.952591756729311</v>
       </c>
       <c r="N10" s="3" t="n">
@@ -1609,17 +1603,17 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0.982162017308068</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.966662811632486</v>
@@ -1628,13 +1622,13 @@
         <v>0.959925387899548</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>0.822597806569674</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0.906070052921289</v>
@@ -1663,19 +1657,19 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0.999815401910504</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0.989382343252623</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0.935886957829521</v>
@@ -1683,22 +1677,22 @@
       <c r="G12" s="3" t="n">
         <v>0.962893870045045</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="I12" s="5" t="n">
+      <c r="H12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I12" s="7" t="n">
         <v>0.9876631841809</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K12" s="5" t="n">
+      <c r="J12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K12" s="7" t="n">
         <v>0.926476657838993</v>
       </c>
-      <c r="L12" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="M12" s="5" t="n">
+      <c r="L12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M12" s="7" t="n">
         <v>0.917914289212563</v>
       </c>
       <c r="N12" s="3" t="n">
@@ -1725,13 +1719,13 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>0.998857575440015</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0.978773666030853</v>
@@ -1741,22 +1735,22 @@
       <c r="G13" s="3" t="n">
         <v>0.952230728471489</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="I13" s="5" t="n">
+      <c r="H13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>0.643835941288096</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="K13" s="5" t="n">
+      <c r="J13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K13" s="7" t="n">
         <v>0.926476657838993</v>
       </c>
-      <c r="L13" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="M13" s="5" t="n">
+      <c r="L13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M13" s="7" t="n">
         <v>0.917914289212563</v>
       </c>
       <c r="N13" s="3" t="n">
@@ -1783,19 +1777,19 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>0.999634904603643</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.993735864660899</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0.974701292029618</v>
@@ -1804,19 +1798,19 @@
         <v>0.992653068077636</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0.98425083967389</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0.976897023628247</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0.944114062752387</v>
@@ -1845,19 +1839,19 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>0.979995410561769</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0.991109179818512</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0.952304857203524</v>
@@ -1866,13 +1860,13 @@
         <v>0.979167892854913</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>0.90990109162069</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>0.938150905951755</v>
@@ -1903,19 +1897,19 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0.999327849666577</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0.959781921115764</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0.943597731896528</v>
@@ -1924,19 +1918,19 @@
         <v>0.963910554065</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0.956434478702747</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>0.988112916730203</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0.963649979956857</v>
@@ -1965,19 +1959,19 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>0.99782601005135</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0.924833526036329</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0.919687678194686</v>
@@ -1986,13 +1980,13 @@
         <v>0.78625199053601</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>0.950816361205194</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>0.913322435705106</v>
@@ -2023,13 +2017,13 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0.967044278173203</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0.859358364302864</v>
@@ -2040,7 +2034,7 @@
         <v>0.802164301740469</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>0.494898779656719</v>
@@ -2073,13 +2067,13 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0.999998063141444</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0.999997101252786</v>
@@ -2090,19 +2084,19 @@
         <v>0.999998769525441</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>0.999770604769915</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>0.964904998960832</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.998558317949646</v>
@@ -2131,13 +2125,13 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0.991716964327734</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0.981915246549224</v>
@@ -2148,19 +2142,19 @@
         <v>0.973035023524191</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>0.957867403100326</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0.945036842348765</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0.953603991510273</v>
@@ -2189,19 +2183,19 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0.997918760549287</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0.987525935953569</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0.98989655845458</v>
@@ -2210,19 +2204,19 @@
         <v>0.984847130391425</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>0.980511641534386</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>0.983749624692239</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0.983749624551454</v>
@@ -2251,38 +2245,38 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0.930234881164427</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>0.975318022177494</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" s="3" t="n">
+      <c r="E22" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" s="5" t="n">
         <v>0.949138309714641</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="2" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>0.797947846170746</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>0.973511853313654</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0.948565989973414</v>
@@ -2309,13 +2303,13 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0.999977796564724</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>0.997152554254249</v>
@@ -2326,13 +2320,13 @@
         <v>0.994759255835993</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>0.99811613478244</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>0.992624380002896</v>
@@ -2363,13 +2357,13 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>1</v>
@@ -2380,13 +2374,13 @@
         <v>1</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>0.94431118528519</v>
@@ -2417,13 +2411,13 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.99902891340686</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0.999098612037334</v>
@@ -2434,13 +2428,13 @@
         <v>0.999651240340044</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>0.998055396153645</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>0.913211851073001</v>
@@ -2471,19 +2465,19 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.997224063407548</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0.990826011212309</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.997866554953488</v>
@@ -2492,13 +2486,13 @@
         <v>0.983277628405395</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0.926638815378631</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0.9748626883743</v>
@@ -2529,13 +2523,13 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.998016917110708</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0.956199772930876</v>
@@ -2545,20 +2539,20 @@
       <c r="G27" s="3" t="n">
         <v>0.903787160547224</v>
       </c>
-      <c r="H27" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="I27" s="5" t="n">
+      <c r="H27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I27" s="7" t="n">
         <v>0.578876004293571</v>
       </c>
-      <c r="J27" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K27" s="5" t="n">
+      <c r="J27" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K27" s="7" t="n">
         <v>0.934723603717686</v>
       </c>
-      <c r="L27" s="4"/>
-      <c r="M27" s="5"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="7"/>
       <c r="N27" s="3" t="n">
         <v>0.583428118931199</v>
       </c>
@@ -2583,13 +2577,13 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.998952350419198</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0.99171174719966</v>
@@ -2599,20 +2593,20 @@
       <c r="G28" s="3" t="n">
         <v>0.982120219990487</v>
       </c>
-      <c r="H28" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="I28" s="5" t="n">
+      <c r="H28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I28" s="7" t="n">
         <v>0.95772281360567</v>
       </c>
-      <c r="J28" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K28" s="5" t="n">
+      <c r="J28" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K28" s="7" t="n">
         <v>0.934723603717686</v>
       </c>
-      <c r="L28" s="4"/>
-      <c r="M28" s="5"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="7"/>
       <c r="N28" s="3" t="n">
         <v>0.949020995879139</v>
       </c>
@@ -2637,13 +2631,13 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.99769796743711</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0.598432829729605</v>
@@ -2653,20 +2647,20 @@
       <c r="G29" s="3" t="n">
         <v>0.567830470268594</v>
       </c>
-      <c r="H29" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="I29" s="5" t="n">
+      <c r="H29" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I29" s="7" t="n">
         <v>0.439321442308408</v>
       </c>
-      <c r="J29" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K29" s="5" t="n">
+      <c r="J29" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K29" s="7" t="n">
         <v>0.934723603717686</v>
       </c>
-      <c r="L29" s="4"/>
-      <c r="M29" s="5"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="7"/>
       <c r="N29" s="3" t="n">
         <v>0.837561394578446</v>
       </c>
@@ -2691,13 +2685,13 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.994265618984518</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>0.960618679596976</v>
@@ -2708,13 +2702,13 @@
         <v>0.926005386424851</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>0.966191991161316</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>0.988733344519805</v>
@@ -2745,38 +2739,38 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.997724733479643</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>0.642466773208739</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F31" s="3" t="n">
+      <c r="E31" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F31" s="5" t="n">
         <v>0.919336320026093</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>0.537837150518689</v>
       </c>
-      <c r="H31" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I31" s="5" t="n">
+      <c r="H31" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="I31" s="7" t="n">
         <v>0.509401386863396</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="M31" s="5" t="n">
+      <c r="J31" s="6"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M31" s="7" t="n">
         <v>0.904943856064789</v>
       </c>
       <c r="N31" s="3" t="n">
@@ -2803,19 +2797,19 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.993433690060039</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>0.928962481361075</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.965491583140523</v>
@@ -2823,18 +2817,18 @@
       <c r="G32" s="3" t="n">
         <v>0.937843010334813</v>
       </c>
-      <c r="H32" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I32" s="5" t="n">
+      <c r="H32" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="I32" s="7" t="n">
         <v>0.90936321357593</v>
       </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="M32" s="5" t="n">
+      <c r="J32" s="6"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M32" s="7" t="n">
         <v>0.904943856064789</v>
       </c>
       <c r="N32" s="3" t="n">
@@ -2861,13 +2855,13 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999703811266792</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>0.985553780843009</v>
@@ -2878,7 +2872,7 @@
         <v>0.971992601692081</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>0.971905124482824</v>
@@ -2911,28 +2905,28 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996123882650309</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0.96979518794634</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F34" s="3" t="n">
+      <c r="E34" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F34" s="5" t="n">
         <v>0.925576196874315</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>0.955939758689639</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>0.803793159228948</v>
@@ -2965,19 +2959,19 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.998480754546317</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>0.992422611199076</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.980296456398047</v>
@@ -2986,19 +2980,19 @@
         <v>0.99559249838149</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.989772746530277</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>0.927074459274781</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0.953409382692888</v>
@@ -3027,13 +3021,13 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.995468844953502</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>0.960943721195381</v>
@@ -3044,7 +3038,7 @@
         <v>0.950982895098882</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>0.773087063383051</v>
@@ -3077,13 +3071,13 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.998932166823345</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0.986810513388783</v>
@@ -3094,19 +3088,19 @@
         <v>0.986570525764206</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>0.936089201810795</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>0.928441807163585</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>164</v>
+        <v>54</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0.986852392055639</v>
@@ -3135,13 +3129,13 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.996905610562691</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0.928329826661788</v>
@@ -3152,7 +3146,7 @@
         <v>0.866109790099055</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>0.645229444653891</v>
@@ -3160,7 +3154,7 @@
       <c r="J38" s="2"/>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0.936729598778588</v>
@@ -3189,13 +3183,13 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.930872311245074</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>0.850413851972058</v>
@@ -3206,7 +3200,7 @@
         <v>0.675995300576774</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>0.746129945546971</v>
@@ -3239,13 +3233,13 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.998465584026839</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>0.995254467621926</v>
@@ -3256,7 +3250,7 @@
         <v>0.997728519333611</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>0.959775759711831</v>
@@ -3264,7 +3258,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0.928952639111837</v>
@@ -3293,13 +3287,13 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.999157789152344</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="D41" s="3" t="n">
         <v>0.998585593823146</v>
@@ -3310,7 +3304,7 @@
         <v>0.993154898603039</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>0.941258954609845</v>
@@ -3343,13 +3337,13 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996471867558548</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>0.984695082908958</v>
@@ -3359,18 +3353,18 @@
       <c r="G42" s="3" t="n">
         <v>0.993773664897899</v>
       </c>
-      <c r="H42" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="I42" s="5" t="n">
+      <c r="H42" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="I42" s="7" t="n">
         <v>0.559632299427059</v>
       </c>
-      <c r="J42" s="4"/>
-      <c r="K42" s="5"/>
-      <c r="L42" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="M42" s="5" t="n">
+      <c r="J42" s="6"/>
+      <c r="K42" s="7"/>
+      <c r="L42" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="M42" s="7" t="n">
         <v>0.991819220378155</v>
       </c>
       <c r="N42" s="3" t="n">
@@ -3397,13 +3391,13 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.995798184879296</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>0.837689830645915</v>
@@ -3413,18 +3407,18 @@
       <c r="G43" s="3" t="n">
         <v>0.852573069055459</v>
       </c>
-      <c r="H43" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="I43" s="5" t="n">
+      <c r="H43" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="I43" s="7" t="n">
         <v>0.289971648819954</v>
       </c>
-      <c r="J43" s="4"/>
-      <c r="K43" s="5"/>
-      <c r="L43" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="M43" s="5" t="n">
+      <c r="J43" s="6"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="M43" s="7" t="n">
         <v>0.991819220378155</v>
       </c>
       <c r="N43" s="3" t="n">
@@ -3451,24 +3445,24 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="2" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>0.66987386568394</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.969213303775499</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.579038811454065</v>
@@ -3499,13 +3493,13 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.992268994192989</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>0.99790446163642</v>
@@ -3516,7 +3510,7 @@
         <v>0.994479470566958</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>0.504211903569637</v>
@@ -3549,13 +3543,13 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.997445021358874</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>0.994483240560779</v>
@@ -3566,7 +3560,7 @@
         <v>0.976652004477945</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>0.92372504933245</v>
@@ -3599,28 +3593,28 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>0.963008094039371</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>0.941081173806262</v>
       </c>
-      <c r="E47" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F47" s="3" t="n">
+      <c r="E47" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F47" s="5" t="n">
         <v>0.93766289313779</v>
       </c>
       <c r="G47" s="3" t="n">
         <v>0.968820362778515</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>0.801500318970652</v>
@@ -3653,19 +3647,19 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>0.993313546180306</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D48" s="3" t="n">
         <v>0.983675304020195</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0.909292168067431</v>
@@ -3674,7 +3668,7 @@
         <v>0.963036985482454</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>0.998475150576667</v>
@@ -3707,7 +3701,12 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>202</v>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed error introduced by editing .tsv files in libreoffice
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -1059,7 +1059,9 @@
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="3" t="n">
+        <v>0.992730200940145</v>
+      </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
@@ -1093,7 +1095,9 @@
       <c r="M2" s="7" t="n">
         <v>0.998577618888331</v>
       </c>
-      <c r="N2" s="3"/>
+      <c r="N2" s="3" t="n">
+        <v>0.997748545019398</v>
+      </c>
       <c r="O2" s="2" t="b">
         <v>0</v>
       </c>
@@ -1107,10 +1111,10 @@
         <v>1</v>
       </c>
       <c r="S2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1118,7 +1122,7 @@
         <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.622786745279133</v>
+        <v>0.995824348751852</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
@@ -1154,7 +1158,7 @@
         <v>0.998577618888331</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.997748545019398</v>
+        <v>0.961495915397195</v>
       </c>
       <c r="O3" s="2" t="b">
         <v>0</v>
@@ -1180,7 +1184,7 @@
         <v>28</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.778580515798629</v>
+        <v>0.961311961936925</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>29</v>
@@ -1216,7 +1220,7 @@
         <v>0.998577618888331</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.961495915397195</v>
+        <v>0.995677422803032</v>
       </c>
       <c r="O4" s="2" t="b">
         <v>0</v>
@@ -1242,7 +1246,7 @@
         <v>31</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.371953933906494</v>
+        <v>0.997816677302374</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>32</v>
@@ -1274,7 +1278,7 @@
         <v>0.998577618888331</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>0.683063690663701</v>
+        <v>0.997650593159154</v>
       </c>
       <c r="O5" s="2" t="b">
         <v>0</v>
@@ -1300,7 +1304,7 @@
         <v>33</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.356219725090913</v>
+        <v>0.980501734047094</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>34</v>
@@ -1336,7 +1340,7 @@
         <v>0.998910219006335</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.0987733626064084</v>
+        <v>0.981043965694831</v>
       </c>
       <c r="O6" s="2" t="b">
         <v>0</v>
@@ -1362,7 +1366,7 @@
         <v>38</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.250049421307193</v>
+        <v>0.985087090067255</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>39</v>
@@ -1394,7 +1398,7 @@
         <v>0.998910219006335</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.981043965694831</v>
+        <v>0.900903588821511</v>
       </c>
       <c r="O7" s="2" t="b">
         <v>0</v>
@@ -1420,7 +1424,7 @@
         <v>40</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.270084198449336</v>
+        <v>0.983098547202523</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>41</v>
@@ -1452,7 +1456,7 @@
         <v>0.998910219006335</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.900903588821511</v>
+        <v>0.987968599664841</v>
       </c>
       <c r="O8" s="2" t="b">
         <v>0</v>
@@ -1478,7 +1482,7 @@
         <v>42</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.152131715392581</v>
+        <v>0.995407107687552</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>43</v>
@@ -1514,7 +1518,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.0924412467549159</v>
+        <v>0.911690781830494</v>
       </c>
       <c r="O9" s="2" t="b">
         <v>0</v>
@@ -1540,7 +1544,7 @@
         <v>47</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.915480914738242</v>
+        <v>0.99886526497977</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>48</v>
@@ -1576,7 +1580,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.911690781830494</v>
+        <v>0.998463405790827</v>
       </c>
       <c r="O10" s="2" t="b">
         <v>0</v>
@@ -1656,7 +1660,7 @@
         <v>55</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.803562829909649</v>
+        <v>0.999815401910504</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>56</v>
@@ -1692,7 +1696,7 @@
         <v>0.917914289212563</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.683596831630516</v>
+        <v>0.998326844708373</v>
       </c>
       <c r="O12" s="2" t="b">
         <v>0</v>
@@ -1718,7 +1722,7 @@
         <v>60</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.833949613195802</v>
+        <v>0.998857575440015</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>61</v>
@@ -1750,7 +1754,7 @@
         <v>0.917914289212563</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.998326844708373</v>
+        <v>0.694378853775062</v>
       </c>
       <c r="O13" s="2" t="b">
         <v>0</v>
@@ -1776,7 +1780,7 @@
         <v>62</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.397800517685714</v>
+        <v>0.999634904603643</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>63</v>
@@ -1812,7 +1816,7 @@
         <v>0.944114062752387</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.319491757898893</v>
+        <v>0.999149430943907</v>
       </c>
       <c r="O14" s="2" t="b">
         <v>0</v>
@@ -1838,7 +1842,7 @@
         <v>67</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.0246072562508828</v>
+        <v>0.979995410561769</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>68</v>
@@ -1870,7 +1874,7 @@
       <c r="L15" s="2"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3" t="n">
-        <v>0.0602052385214646</v>
+        <v>0.150045204780609</v>
       </c>
       <c r="O15" s="2" t="b">
         <v>1</v>
@@ -1896,7 +1900,7 @@
         <v>72</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.02160584886913</v>
+        <v>0.999327849666577</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>73</v>
@@ -1932,7 +1936,7 @@
         <v>0.963649979956857</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.0513811514674906</v>
+        <v>0.997720094826182</v>
       </c>
       <c r="O16" s="2" t="b">
         <v>0</v>
@@ -1958,7 +1962,7 @@
         <v>77</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.224993902268702</v>
+        <v>0.99782601005135</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>78</v>
@@ -1990,7 +1994,7 @@
       <c r="L17" s="2"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3" t="n">
-        <v>0.214080123720895</v>
+        <v>0.979763131510324</v>
       </c>
       <c r="O17" s="2" t="b">
         <v>0</v>
@@ -2016,7 +2020,7 @@
         <v>82</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.302978486935989</v>
+        <v>0.967044278173203</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>83</v>
@@ -2040,7 +2044,7 @@
       <c r="L18" s="2"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3" t="n">
-        <v>0.273300448549736</v>
+        <v>0.886500375872699</v>
       </c>
       <c r="O18" s="2" t="b">
         <v>1</v>
@@ -2066,7 +2070,7 @@
         <v>85</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.13933865879166</v>
+        <v>0.999998063141444</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>86</v>
@@ -2098,7 +2102,7 @@
         <v>0.998558317949646</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.166459682383803</v>
+        <v>0.999823035936981</v>
       </c>
       <c r="O19" s="2" t="b">
         <v>0</v>
@@ -2124,7 +2128,7 @@
         <v>90</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.0243223615828175</v>
+        <v>0.991716964327734</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>91</v>
@@ -2156,7 +2160,7 @@
         <v>0.953603991510273</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.0826748223160879</v>
+        <v>0.210290293749863</v>
       </c>
       <c r="O20" s="2" t="b">
         <v>0</v>
@@ -2182,7 +2186,7 @@
         <v>94</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.103673748658306</v>
+        <v>0.188996063535915</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>95</v>
@@ -2218,7 +2222,7 @@
         <v>0.983749624551454</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.15488511546483</v>
+        <v>0.194386082170664</v>
       </c>
       <c r="O21" s="2" t="b">
         <v>0</v>
@@ -2300,7 +2304,7 @@
         <v>104</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.108005395671567</v>
+        <v>0.999977796564724</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>105</v>
@@ -2328,7 +2332,7 @@
       <c r="L23" s="2"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3" t="n">
-        <v>0.1450294727464</v>
+        <v>0.999989282192406</v>
       </c>
       <c r="O23" s="2" t="b">
         <v>0</v>
@@ -2354,7 +2358,7 @@
         <v>108</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>109</v>
@@ -2382,7 +2386,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3" t="n">
-        <v>0</v>
+        <v>0.672733978438699</v>
       </c>
       <c r="O24" s="2" t="b">
         <v>0</v>
@@ -2408,7 +2412,7 @@
         <v>112</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0.171449968800704</v>
+        <v>0.99902891340686</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>113</v>
@@ -2436,7 +2440,7 @@
       <c r="L25" s="2"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3" t="n">
-        <v>0.101401017909111</v>
+        <v>0.994357056665344</v>
       </c>
       <c r="O25" s="2" t="b">
         <v>0</v>
@@ -2462,7 +2466,7 @@
         <v>116</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.0574735080140215</v>
+        <v>0.997224063407548</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>117</v>
@@ -2494,7 +2498,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3" t="n">
-        <v>0.121536117910536</v>
+        <v>0.966490093087254</v>
       </c>
       <c r="O26" s="2" t="b">
         <v>0</v>
@@ -2520,7 +2524,7 @@
         <v>121</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.213388214879899</v>
+        <v>0.998016917110708</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>122</v>
@@ -2548,7 +2552,7 @@
       <c r="L27" s="6"/>
       <c r="M27" s="7"/>
       <c r="N27" s="3" t="n">
-        <v>0.11646234804336</v>
+        <v>0.583428118931199</v>
       </c>
       <c r="O27" s="2" t="b">
         <v>0</v>
@@ -2574,7 +2578,7 @@
         <v>125</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.751484788877061</v>
+        <v>0.998952350419198</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>126</v>
@@ -2602,7 +2606,7 @@
       <c r="L28" s="6"/>
       <c r="M28" s="7"/>
       <c r="N28" s="3" t="n">
-        <v>0.583428118931199</v>
+        <v>0.949020995879139</v>
       </c>
       <c r="O28" s="2" t="b">
         <v>0</v>
@@ -2628,7 +2632,7 @@
         <v>127</v>
       </c>
       <c r="B29" s="3" t="n">
-        <v>0.782430695535662</v>
+        <v>0.99769796743711</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>128</v>
@@ -2656,7 +2660,7 @@
       <c r="L29" s="6"/>
       <c r="M29" s="7"/>
       <c r="N29" s="3" t="n">
-        <v>0.949020995879139</v>
+        <v>0.837561394578446</v>
       </c>
       <c r="O29" s="2" t="b">
         <v>0</v>
@@ -2682,7 +2686,7 @@
         <v>129</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>0.127288634336652</v>
+        <v>0.994265618984518</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>130</v>
@@ -2710,7 +2714,7 @@
       <c r="L30" s="2"/>
       <c r="M30" s="3"/>
       <c r="N30" s="3" t="n">
-        <v>0.144734835834405</v>
+        <v>0.990644897191167</v>
       </c>
       <c r="O30" s="2" t="b">
         <v>0</v>
@@ -2736,7 +2740,7 @@
         <v>133</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>0.31257386282561</v>
+        <v>0.997724733479643</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>134</v>
@@ -2768,7 +2772,7 @@
         <v>0.904943856064789</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>0.377992966753821</v>
+        <v>0.996416507294122</v>
       </c>
       <c r="O31" s="2" t="b">
         <v>0</v>
@@ -2794,7 +2798,7 @@
         <v>137</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>0.908635935389673</v>
+        <v>0.993433690060039</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>138</v>
@@ -2826,7 +2830,7 @@
         <v>0.904943856064789</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>0.996416507294122</v>
+        <v>0.954279690330215</v>
       </c>
       <c r="O32" s="2" t="b">
         <v>0</v>
@@ -2852,7 +2856,7 @@
         <v>140</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.296850405329504</v>
+        <v>0.999703811266792</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>141</v>
@@ -2876,7 +2880,7 @@
       <c r="L33" s="2"/>
       <c r="M33" s="3"/>
       <c r="N33" s="3" t="n">
-        <v>0.346852244892979</v>
+        <v>0.99665835952651</v>
       </c>
       <c r="O33" s="2" t="b">
         <v>0</v>
@@ -2902,7 +2906,7 @@
         <v>143</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.252226268708498</v>
+        <v>0.996123882650309</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>144</v>
@@ -2930,7 +2934,7 @@
       <c r="L34" s="2"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3" t="n">
-        <v>0.35916395227216</v>
+        <v>0.888842583261856</v>
       </c>
       <c r="O34" s="2" t="b">
         <v>0</v>
@@ -2956,7 +2960,7 @@
         <v>147</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0.138700611715243</v>
+        <v>0.998480754546317</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>148</v>
@@ -2992,7 +2996,7 @@
         <v>0.953409382692888</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.203101108317241</v>
+        <v>0.98781745464669</v>
       </c>
       <c r="O35" s="2" t="b">
         <v>0</v>
@@ -3018,7 +3022,7 @@
         <v>151</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.220003710971997</v>
+        <v>0.995468844953502</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>152</v>
@@ -3042,7 +3046,7 @@
       <c r="L36" s="2"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3" t="n">
-        <v>0.789015917379536</v>
+        <v>0.981035375612377</v>
       </c>
       <c r="O36" s="2" t="b">
         <v>0</v>
@@ -3068,7 +3072,7 @@
         <v>154</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>0.077369263913022</v>
+        <v>0.998932166823345</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>155</v>
@@ -3100,7 +3104,7 @@
         <v>0.986852392055639</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>0.1078954165964</v>
+        <v>0.995222320803457</v>
       </c>
       <c r="O37" s="2" t="b">
         <v>0</v>
@@ -3126,7 +3130,7 @@
         <v>157</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>0.0740517666785148</v>
+        <v>0.996905610562691</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>158</v>
@@ -3154,7 +3158,7 @@
         <v>0.936729598778588</v>
       </c>
       <c r="N38" s="3" t="n">
-        <v>0.064787618761053</v>
+        <v>0.956288683422495</v>
       </c>
       <c r="O38" s="2" t="b">
         <v>0</v>
@@ -3180,7 +3184,7 @@
         <v>161</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.111531967685043</v>
+        <v>0.930872311245074</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>162</v>
@@ -3204,7 +3208,7 @@
       <c r="L39" s="2"/>
       <c r="M39" s="3"/>
       <c r="N39" s="3" t="n">
-        <v>0.156471712418937</v>
+        <v>0.819795871635397</v>
       </c>
       <c r="O39" s="2" t="b">
         <v>0</v>
@@ -3230,7 +3234,7 @@
         <v>164</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>0.127866377402439</v>
+        <v>0.998465584026839</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>165</v>
@@ -3258,7 +3262,7 @@
         <v>0.928952639111837</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>0.141175739712967</v>
+        <v>0.983807389953579</v>
       </c>
       <c r="O40" s="2" t="b">
         <v>0</v>
@@ -3284,7 +3288,7 @@
         <v>168</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0.0552618298350718</v>
+        <v>0.999157789152344</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>169</v>
@@ -3308,7 +3312,7 @@
       <c r="L41" s="2"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3" t="n">
-        <v>0.0436560704588343</v>
+        <v>0.0573439955343392</v>
       </c>
       <c r="O41" s="2" t="b">
         <v>1</v>
@@ -3334,7 +3338,7 @@
         <v>171</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>0.222535263892146</v>
+        <v>0.996471867558548</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>172</v>
@@ -3362,7 +3366,7 @@
         <v>0.991819220378155</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>0.103952273544675</v>
+        <v>0.557852701797722</v>
       </c>
       <c r="O42" s="2" t="b">
         <v>0</v>
@@ -3388,7 +3392,7 @@
         <v>175</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>0.732601177765574</v>
+        <v>0.995798184879296</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>176</v>
@@ -3416,7 +3420,7 @@
         <v>0.991819220378155</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>0.557852701797722</v>
+        <v>0.547301794595584</v>
       </c>
       <c r="O43" s="2" t="b">
         <v>0</v>
@@ -3490,7 +3494,7 @@
         <v>181</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>0.111722228670123</v>
+        <v>0.992268994192989</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>182</v>
@@ -3514,7 +3518,7 @@
       <c r="L45" s="2"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3" t="n">
-        <v>0.157225439773526</v>
+        <v>0.587167215139279</v>
       </c>
       <c r="O45" s="2" t="b">
         <v>0</v>
@@ -3540,7 +3544,7 @@
         <v>184</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>0.385923046323566</v>
+        <v>0.997445021358874</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>185</v>
@@ -3564,7 +3568,7 @@
       <c r="L46" s="2"/>
       <c r="M46" s="3"/>
       <c r="N46" s="3" t="n">
-        <v>0.110735505529089</v>
+        <v>0.0475462843338336</v>
       </c>
       <c r="O46" s="2" t="b">
         <v>1</v>
@@ -3590,7 +3594,7 @@
         <v>187</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>0.0984003147259527</v>
+        <v>0.963008094039371</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>188</v>
@@ -3618,7 +3622,7 @@
       <c r="L47" s="2"/>
       <c r="M47" s="3"/>
       <c r="N47" s="3" t="n">
-        <v>0.0571567009172643</v>
+        <v>0.102429900117076</v>
       </c>
       <c r="O47" s="2" t="b">
         <v>1</v>
@@ -3644,7 +3648,7 @@
         <v>191</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>0.73005839696477</v>
+        <v>0.993313546180306</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>192</v>
@@ -3672,7 +3676,7 @@
       <c r="L48" s="2"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3" t="n">
-        <v>0.839870005998011</v>
+        <v>0.986654622703124</v>
       </c>
       <c r="O48" s="2" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
re-ran plot_si... asignment and vigentte.qmd
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -1060,19 +1060,19 @@
         <v>20</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.992730200940145</v>
+        <v>0.992730200825371</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.980247231981805</v>
+        <v>0.980247231701711</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.982523066590154</v>
+        <v>0.982523066261465</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0.9596639524824</v>
@@ -1122,19 +1122,19 @@
         <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.995824348751852</v>
+        <v>0.995824348902905</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.987184801324652</v>
+        <v>0.987184800818609</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.961293866458291</v>
+        <v>0.96129386656296</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>0.971169546248927</v>
@@ -1184,19 +1184,19 @@
         <v>28</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.961311961936925</v>
+        <v>0.961311962410772</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.923032940882415</v>
+        <v>0.923032940814617</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>30</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.93647989440547</v>
+        <v>0.936479893911556</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0.929054257037847</v>
@@ -1246,13 +1246,13 @@
         <v>31</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.997816677302374</v>
+        <v>0.997816677276983</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.99675737544784</v>
+        <v>0.996757375473159</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
@@ -1304,19 +1304,19 @@
         <v>33</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.980501734047094</v>
+        <v>0.980501733856783</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.990263031835387</v>
+        <v>0.990263031998398</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>35</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.905687533553426</v>
+        <v>0.905687534023291</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0.967949920301316</v>
@@ -1366,13 +1366,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.985087090067255</v>
+        <v>0.985087089697391</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.933667457882778</v>
+        <v>0.933667457212448</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
@@ -1424,13 +1424,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.983098547202523</v>
+        <v>0.983098546742857</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.979438082042213</v>
+        <v>0.979438081432212</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
@@ -1482,19 +1482,19 @@
         <v>42</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.995407107687552</v>
+        <v>0.995407108006126</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>43</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.953117492152762</v>
+        <v>0.953117493420828</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>44</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.913569151804241</v>
+        <v>0.913569151516943</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>0.893003527564203</v>
@@ -1544,19 +1544,19 @@
         <v>47</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.99886526497977</v>
+        <v>0.998865265130157</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.992284649786581</v>
+        <v>0.992284650997823</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>49</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.953522795429812</v>
+        <v>0.953522795453119</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0.990426082637624</v>
@@ -1610,13 +1610,13 @@
         <v>51</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.982162017308068</v>
+        <v>0.982162017701685</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.966662811632486</v>
+        <v>0.966662811925343</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>0.959925387899548</v>
@@ -1660,19 +1660,19 @@
         <v>55</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.999815401910504</v>
+        <v>0.999815401416271</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>56</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.989382343252623</v>
+        <v>0.98938234008859</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>57</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.935886957829521</v>
+        <v>0.935886952837027</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0.962893870045045</v>
@@ -1722,13 +1722,13 @@
         <v>60</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.998857575440015</v>
+        <v>0.998857574204807</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>61</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.978773666030853</v>
+        <v>0.978773665116604</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
@@ -1780,19 +1780,19 @@
         <v>62</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.999634904603643</v>
+        <v>0.999634904581738</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>63</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.993735864660899</v>
+        <v>0.993735864518384</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>64</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.974701292029618</v>
+        <v>0.974701291825274</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0.992653068077636</v>
@@ -1842,19 +1842,19 @@
         <v>67</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.979995410561769</v>
+        <v>0.979995410562213</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.991109179818512</v>
+        <v>0.991109179393785</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>69</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.952304857203524</v>
+        <v>0.952304859229673</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>0.979167892854913</v>
@@ -1900,19 +1900,19 @@
         <v>72</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.999327849666577</v>
+        <v>0.999327849638883</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.959781921115764</v>
+        <v>0.959781921008911</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>74</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.943597731896528</v>
+        <v>0.943597731745337</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0.963910554065</v>
@@ -1962,19 +1962,19 @@
         <v>77</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.99782601005135</v>
+        <v>0.997826010088387</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.924833526036329</v>
+        <v>0.924833525763961</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>79</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.919687678194686</v>
+        <v>0.919687679199628</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>0.78625199053601</v>
@@ -2020,13 +2020,13 @@
         <v>82</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.967044278173203</v>
+        <v>0.967044279115935</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.859358364302864</v>
+        <v>0.859358363501512</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
@@ -2070,13 +2070,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.999998063141444</v>
+        <v>0.999998063141562</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.999997101252786</v>
+        <v>0.99999710125291</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
@@ -2128,13 +2128,13 @@
         <v>90</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.991716964327734</v>
+        <v>0.991716964217417</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>91</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.981915246549224</v>
+        <v>0.9819152461787</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
@@ -2186,19 +2186,19 @@
         <v>94</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.188996063535915</v>
+        <v>0.188996059832515</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.987525935953569</v>
+        <v>0.987525936035042</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>96</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.98989655845458</v>
+        <v>0.989896555611974</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>0.984847130391425</v>
@@ -2252,13 +2252,13 @@
         <v>100</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.975318022177494</v>
+        <v>0.975318022355795</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>101</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.949138309714641</v>
+        <v>0.949138309746127</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="2" t="s">
@@ -2304,13 +2304,13 @@
         <v>104</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.999977796564724</v>
+        <v>0.999977796576728</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>105</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.997152554254249</v>
+        <v>0.997152554293266</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
@@ -2412,13 +2412,13 @@
         <v>112</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0.99902891340686</v>
+        <v>0.999028913454499</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>113</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.999098612037334</v>
+        <v>0.999098612098447</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
@@ -2466,19 +2466,19 @@
         <v>116</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.997224063407548</v>
+        <v>0.997224063445585</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>117</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.990826011212309</v>
+        <v>0.990826011162356</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>118</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.997866554953488</v>
+        <v>0.997866554870421</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>0.983277628405395</v>
@@ -2524,13 +2524,13 @@
         <v>121</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.998016917110708</v>
+        <v>0.998016917127346</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>122</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.956199772930876</v>
+        <v>0.956199773890916</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
@@ -2578,13 +2578,13 @@
         <v>125</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.998952350419198</v>
+        <v>0.998952350407319</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>126</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.99171174719966</v>
+        <v>0.991711747199947</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="3"/>
@@ -2632,13 +2632,13 @@
         <v>127</v>
       </c>
       <c r="B29" s="3" t="n">
-        <v>0.99769796743711</v>
+        <v>0.997697967449371</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>128</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.598432829729605</v>
+        <v>0.59843282958418</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="3"/>
@@ -2686,13 +2686,13 @@
         <v>129</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>0.994265618984518</v>
+        <v>0.994265618936021</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>130</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.960618679596976</v>
+        <v>0.960618679377363</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="3"/>
@@ -2740,19 +2740,19 @@
         <v>133</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>0.997724733479643</v>
+        <v>0.997724733557505</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>134</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.642466773208739</v>
+        <v>0.642466773271259</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>135</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.919336320026093</v>
+        <v>0.919336320629207</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>0.537837150518689</v>
@@ -2798,19 +2798,19 @@
         <v>137</v>
       </c>
       <c r="B32" s="3" t="n">
-        <v>0.993433690060039</v>
+        <v>0.993433690246823</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>138</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.928962481361075</v>
+        <v>0.928962481898069</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>139</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0.965491583140523</v>
+        <v>0.965491583372847</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>0.937843010334813</v>
@@ -2856,13 +2856,13 @@
         <v>140</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.999703811266792</v>
+        <v>0.999703811227718</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>141</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.985553780843009</v>
+        <v>0.985553780930321</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" s="3"/>
@@ -2906,19 +2906,19 @@
         <v>143</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.996123882650309</v>
+        <v>0.996123882583084</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>144</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0.96979518794634</v>
+        <v>0.969795188277553</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>145</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.925576196874315</v>
+        <v>0.925576196292447</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>0.955939758689639</v>
@@ -2960,19 +2960,19 @@
         <v>147</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0.998480754546317</v>
+        <v>0.998480754546849</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>148</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.992422611199076</v>
+        <v>0.992422611149915</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>149</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0.980296456398047</v>
+        <v>0.980296456463297</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>0.99559249838149</v>
@@ -3022,13 +3022,13 @@
         <v>151</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.995468844953502</v>
+        <v>0.99546884480786</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>152</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0.960943721195381</v>
+        <v>0.960943720955395</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="3"/>
@@ -3072,13 +3072,13 @@
         <v>154</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>0.998932166823345</v>
+        <v>0.998932166853944</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>155</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.986810513388783</v>
+        <v>0.986810513377358</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="3"/>
@@ -3130,13 +3130,13 @@
         <v>157</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>0.996905610562691</v>
+        <v>0.996905610452122</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>158</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.928329826661788</v>
+        <v>0.928329826828612</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="3"/>
@@ -3184,13 +3184,13 @@
         <v>161</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.930872311245074</v>
+        <v>0.930872311433532</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>162</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.850413851972058</v>
+        <v>0.85041385190883</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="3"/>
@@ -3234,13 +3234,13 @@
         <v>164</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>0.998465584026839</v>
+        <v>0.998465583966881</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>165</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.995254467621926</v>
+        <v>0.995254467848528</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" s="3"/>
@@ -3288,13 +3288,13 @@
         <v>168</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0.999157789152344</v>
+        <v>0.99915778915087</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>169</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>0.998585593823146</v>
+        <v>0.998585593777231</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" s="3"/>
@@ -3338,13 +3338,13 @@
         <v>171</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>0.996471867558548</v>
+        <v>0.996471867499297</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>172</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.984695082908958</v>
+        <v>0.984695082690026</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" s="3"/>
@@ -3392,13 +3392,13 @@
         <v>175</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>0.995798184879296</v>
+        <v>0.995798184740579</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>176</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.837689830645915</v>
+        <v>0.837689830729731</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" s="3"/>
@@ -3450,13 +3450,13 @@
         <v>178</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>0.66987386568394</v>
+        <v>0.669873865803624</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>179</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.969213303775499</v>
+        <v>0.969213303626853</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="2" t="s">
@@ -3494,13 +3494,13 @@
         <v>181</v>
       </c>
       <c r="B45" s="3" t="n">
-        <v>0.992268994192989</v>
+        <v>0.992268993693795</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>182</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.99790446163642</v>
+        <v>0.997904461563255</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" s="3"/>
@@ -3544,13 +3544,13 @@
         <v>184</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>0.997445021358874</v>
+        <v>0.997445021406782</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>185</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.994483240560779</v>
+        <v>0.994483240276513</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" s="3"/>
@@ -3594,19 +3594,19 @@
         <v>187</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>0.963008094039371</v>
+        <v>0.963008093248055</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>188</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.941081173806262</v>
+        <v>0.941081172920484</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>189</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.93766289313779</v>
+        <v>0.937662887460793</v>
       </c>
       <c r="G47" s="3" t="n">
         <v>0.968820362778515</v>
@@ -3648,19 +3648,19 @@
         <v>191</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>0.993313546180306</v>
+        <v>0.993313545860852</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>192</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.983675304020195</v>
+        <v>0.983675304699237</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>193</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>0.909292168067431</v>
+        <v>0.909292167040706</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0.963036985482454</v>

</xml_diff>

<commit_message>
cleaned up table headers; changed 'supporting tumor' to 'linking tumor'
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,66 +12,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="197">
-  <si>
-    <t xml:space="preserve">signature id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sig89 from 476 v 89 cos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">exemplar id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sig89 v exemplar cos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">best match koh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cos v koh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sig476 v exemplar cos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type83 sig id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sig83 v exemplar cos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">best match cosmic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cosine v cosmic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">best match jin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cosine v jin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sig83 from 476 v 83 cos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is polyT removed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is insdel15 16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">has 476 signature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">has 83 signature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">has mapped 476 sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">has 83 mapped signature</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
+  <si>
+    <t xml:space="preserve">signature_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sig89_from_476_v_89_cos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exemplar_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sig89_v_exemplar_cos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best_match_koh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cos_v_koh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sig476_v_exemplar_cos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">type83_sig_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sig83_v_exemplar_cos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best_match_cosmic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cosine_v_cosmic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best_match_jin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cosine_v_jin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sig83_from_476_v_83_cos</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel1a</t>
@@ -599,10 +581,52 @@
     <t xml:space="preserve">ID_P</t>
   </si>
   <si>
-    <t xml:space="preserve">* This is the signature with the best match to the given signature_id.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">** indicates that in the supporting tumor's spectrum, insertions of a single T in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
+    <t xml:space="preserve">Type 89 Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim vs Type 476 Sig Collapsed to Type 89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linking Tumor ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim vs Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best Match to Koh et al., 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim vs Koh et al.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim of Extracted 476-Type Sig vs Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extracted Type-83 Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim of Extracted 83-Type Sig vs Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest COSMIC Sig ID to Extracted 83-Type Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim of COSMIC Sig vs Extracted 83-Type Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest Sig from Jin et al., 2024 to Extracted 83-Type Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim of Jin et al. to Extracted 83-Type Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine Sim vs Type 476 Sig Approx Collapsed to Type 83</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* This is the signature with the best match to the given type-89 signature.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">** indicates that in the supporting tumor's spectrum, insertions of single Ts in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
   </si>
 </sst>
 </file>
@@ -985,91 +1009,67 @@
     <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="8.71" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="7.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="7.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="7.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="6.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="7.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="7.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>190</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>191</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>192</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>193</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>194</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>195</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>196</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>197</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>198</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>199</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>200</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>201</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>0.992730200825371</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0.980247231701711</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.982523066261465</v>
@@ -1078,19 +1078,19 @@
         <v>0.9596639524824</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I2" s="7" t="n">
         <v>0.998418245662758</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>0.998577618888331</v>
@@ -1098,40 +1098,22 @@
       <c r="N2" s="3" t="n">
         <v>0.997748545019398</v>
       </c>
-      <c r="O2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.995824348902905</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0.987184800818609</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.96129386656296</v>
@@ -1140,19 +1122,19 @@
         <v>0.971169546248927</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>0.961390178570747</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>0.998577618888331</v>
@@ -1160,40 +1142,22 @@
       <c r="N3" s="3" t="n">
         <v>0.961495915397195</v>
       </c>
-      <c r="O3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.961311962410772</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0.923032940814617</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.936479893911556</v>
@@ -1202,19 +1166,19 @@
         <v>0.929054257037847</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I4" s="7" t="n">
         <v>0.998493112709776</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>0.998577618888331</v>
@@ -1222,34 +1186,16 @@
       <c r="N4" s="3" t="n">
         <v>0.995677422803032</v>
       </c>
-      <c r="O4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T4" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.997816677276983</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0.996757375473159</v>
@@ -1260,19 +1206,19 @@
         <v>0.994594220752138</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>0.99606877275794</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>0.998997225071613</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>0.998577618888331</v>
@@ -1280,40 +1226,22 @@
       <c r="N5" s="3" t="n">
         <v>0.997650593159154</v>
       </c>
-      <c r="O5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T5" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.980501733856783</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.990263031998398</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0.905687534023291</v>
@@ -1322,19 +1250,19 @@
         <v>0.967949920301316</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>0.896138732515832</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>0.998910219006335</v>
@@ -1342,34 +1270,16 @@
       <c r="N6" s="3" t="n">
         <v>0.981043965694831</v>
       </c>
-      <c r="O6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.985087089697391</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0.933667457212448</v>
@@ -1380,19 +1290,19 @@
         <v>0.931852177125591</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>0.955583423187771</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>0.998910219006335</v>
@@ -1400,34 +1310,16 @@
       <c r="N7" s="3" t="n">
         <v>0.900903588821511</v>
       </c>
-      <c r="O7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0.983098546742857</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0.979438081432212</v>
@@ -1438,19 +1330,19 @@
         <v>0.999362829413946</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>0.982691257770152</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>0.997328276109875</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>0.998910219006335</v>
@@ -1458,40 +1350,22 @@
       <c r="N8" s="3" t="n">
         <v>0.987968599664841</v>
       </c>
-      <c r="O8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.995407108006126</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0.953117493420828</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0.913569151516943</v>
@@ -1500,19 +1374,19 @@
         <v>0.893003527564203</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.90592938388244</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>0.992673228868062</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>0.952591756729311</v>
@@ -1520,40 +1394,22 @@
       <c r="N9" s="3" t="n">
         <v>0.911690781830494</v>
       </c>
-      <c r="O9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P9" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.998865265130157</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.992284650997823</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0.953522795453119</v>
@@ -1562,19 +1418,19 @@
         <v>0.990426082637624</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>0.988504232948747</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>0.992673228868062</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>0.952591756729311</v>
@@ -1582,38 +1438,20 @@
       <c r="N10" s="3" t="n">
         <v>0.998463405790827</v>
       </c>
-      <c r="O10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P10" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0.982162017701685</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.966662811925343</v>
@@ -1622,13 +1460,13 @@
         <v>0.959925387899548</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>0.822597806569674</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0.906070052921289</v>
@@ -1636,40 +1474,22 @@
       <c r="L11" s="2"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
-      <c r="O11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S11" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T11" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0.999815401416271</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0.98938234008859</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0.935886952837027</v>
@@ -1678,19 +1498,19 @@
         <v>0.962893870045045</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>0.9876631841809</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>0.926476657838993</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>0.917914289212563</v>
@@ -1698,34 +1518,16 @@
       <c r="N12" s="3" t="n">
         <v>0.998326844708373</v>
       </c>
-      <c r="O12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>0.998857574204807</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0.978773665116604</v>
@@ -1736,19 +1538,19 @@
         <v>0.952230728471489</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0.643835941288096</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>0.926476657838993</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="M13" s="7" t="n">
         <v>0.917914289212563</v>
@@ -1756,40 +1558,22 @@
       <c r="N13" s="3" t="n">
         <v>0.694378853775062</v>
       </c>
-      <c r="O13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T13" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>0.999634904581738</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.993735864518384</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0.974701291825274</v>
@@ -1798,19 +1582,19 @@
         <v>0.992653068077636</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>0.98425083967389</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>0.976897023628247</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>0.944114062752387</v>
@@ -1818,40 +1602,22 @@
       <c r="N14" s="3" t="n">
         <v>0.999149430943907</v>
       </c>
-      <c r="O14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T14" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>0.979995410562213</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0.991109179393785</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0.952304859229673</v>
@@ -1860,13 +1626,13 @@
         <v>0.979167892854913</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>0.90990109162069</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>0.938150905951755</v>
@@ -1876,40 +1642,22 @@
       <c r="N15" s="3" t="n">
         <v>0.150045204780609</v>
       </c>
-      <c r="O15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T15" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0.999327849638883</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0.959781921008911</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0.943597731745337</v>
@@ -1918,19 +1666,19 @@
         <v>0.963910554065</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>0.956434478702747</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>0.988112916730203</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0.963649979956857</v>
@@ -1938,40 +1686,22 @@
       <c r="N16" s="3" t="n">
         <v>0.997720094826182</v>
       </c>
-      <c r="O16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T16" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>0.997826010088387</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0.924833525763961</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0.919687679199628</v>
@@ -1980,13 +1710,13 @@
         <v>0.78625199053601</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>0.950816361205194</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>0.913322435705106</v>
@@ -1996,34 +1726,16 @@
       <c r="N17" s="3" t="n">
         <v>0.979763131510324</v>
       </c>
-      <c r="O17" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P17" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T17" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0.967044279115935</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0.859358363501512</v>
@@ -2034,7 +1746,7 @@
         <v>0.802164301740469</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>0.494898779656719</v>
@@ -2046,34 +1758,16 @@
       <c r="N18" s="3" t="n">
         <v>0.886500375872699</v>
       </c>
-      <c r="O18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P18" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T18" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0.999998063141562</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0.99999710125291</v>
@@ -2084,19 +1778,19 @@
         <v>0.999998769525441</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>0.999770604769915</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>0.964904998960832</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.998558317949646</v>
@@ -2104,34 +1798,16 @@
       <c r="N19" s="3" t="n">
         <v>0.999823035936981</v>
       </c>
-      <c r="O19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T19" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0.991716964217417</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0.9819152461787</v>
@@ -2142,19 +1818,19 @@
         <v>0.973035023524191</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>0.957867403100326</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>0.945036842348765</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0.953603991510273</v>
@@ -2162,40 +1838,22 @@
       <c r="N20" s="3" t="n">
         <v>0.210290293749863</v>
       </c>
-      <c r="O20" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P20" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T20" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0.188996059832515</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0.987525936035042</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0.989896555611974</v>
@@ -2204,19 +1862,19 @@
         <v>0.984847130391425</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>0.980511641534386</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>0.983749624692239</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>0.983749624551454</v>
@@ -2224,90 +1882,54 @@
       <c r="N21" s="3" t="n">
         <v>0.194386082170664</v>
       </c>
-      <c r="O21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P21" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T21" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>0.975318022355795</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.949138309746127</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>0.797947846170746</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>0.973511853313654</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>0.948565989973414</v>
       </c>
       <c r="N22" s="3"/>
-      <c r="O22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S22" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T22" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0.999977796576728</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>0.997152554293266</v>
@@ -2318,13 +1940,13 @@
         <v>0.994759255835993</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>0.99811613478244</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>0.992624380002896</v>
@@ -2334,34 +1956,16 @@
       <c r="N23" s="3" t="n">
         <v>0.999989282192406</v>
       </c>
-      <c r="O23" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T23" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>1</v>
@@ -2372,13 +1976,13 @@
         <v>1</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>0.94431118528519</v>
@@ -2388,34 +1992,16 @@
       <c r="N24" s="3" t="n">
         <v>0.672733978438699</v>
       </c>
-      <c r="O24" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T24" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.999028913454499</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0.999098612098447</v>
@@ -2426,13 +2012,13 @@
         <v>0.999651240340044</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>0.998055396153645</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>0.913211851073001</v>
@@ -2442,40 +2028,22 @@
       <c r="N25" s="3" t="n">
         <v>0.994357056665344</v>
       </c>
-      <c r="O25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P25" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T25" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.997224063445585</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0.990826011162356</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.997866554870421</v>
@@ -2484,13 +2052,13 @@
         <v>0.983277628405395</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0.926638815378631</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0.9748626883743</v>
@@ -2500,34 +2068,16 @@
       <c r="N26" s="3" t="n">
         <v>0.966490093087254</v>
       </c>
-      <c r="O26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T26" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.998016917127346</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0.956199773890916</v>
@@ -2538,13 +2088,13 @@
         <v>0.903787160547224</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.578876004293571</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2554,34 +2104,16 @@
       <c r="N27" s="3" t="n">
         <v>0.583428118931199</v>
       </c>
-      <c r="O27" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P27" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T27" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.998952350407319</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0.991711747199947</v>
@@ -2592,13 +2124,13 @@
         <v>0.982120219990487</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>0.95772281360567</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2608,34 +2140,16 @@
       <c r="N28" s="3" t="n">
         <v>0.949020995879139</v>
       </c>
-      <c r="O28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T28" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.997697967449371</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0.59843282958418</v>
@@ -2646,13 +2160,13 @@
         <v>0.567830470268594</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.439321442308408</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2662,34 +2176,16 @@
       <c r="N29" s="3" t="n">
         <v>0.837561394578446</v>
       </c>
-      <c r="O29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T29" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.994265618936021</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>0.960618679377363</v>
@@ -2700,13 +2196,13 @@
         <v>0.926005386424851</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>0.966191991161316</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>0.988733344519805</v>
@@ -2716,40 +2212,22 @@
       <c r="N30" s="3" t="n">
         <v>0.990644897191167</v>
       </c>
-      <c r="O30" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P30" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T30" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.997724733557505</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>0.642466773271259</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>0.919336320629207</v>
@@ -2758,7 +2236,7 @@
         <v>0.537837150518689</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.509401386863396</v>
@@ -2766,7 +2244,7 @@
       <c r="J31" s="6"/>
       <c r="K31" s="7"/>
       <c r="L31" s="6" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="M31" s="7" t="n">
         <v>0.904943856064789</v>
@@ -2774,40 +2252,22 @@
       <c r="N31" s="3" t="n">
         <v>0.996416507294122</v>
       </c>
-      <c r="O31" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P31" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T31" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.993433690246823</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>0.928962481898069</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.965491583372847</v>
@@ -2816,7 +2276,7 @@
         <v>0.937843010334813</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="I32" s="7" t="n">
         <v>0.90936321357593</v>
@@ -2824,7 +2284,7 @@
       <c r="J32" s="6"/>
       <c r="K32" s="7"/>
       <c r="L32" s="6" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="M32" s="7" t="n">
         <v>0.904943856064789</v>
@@ -2832,34 +2292,16 @@
       <c r="N32" s="3" t="n">
         <v>0.954279690330215</v>
       </c>
-      <c r="O32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T32" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999703811227718</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>0.985553780930321</v>
@@ -2870,7 +2312,7 @@
         <v>0.971992601692081</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>0.971905124482824</v>
@@ -2882,40 +2324,22 @@
       <c r="N33" s="3" t="n">
         <v>0.99665835952651</v>
       </c>
-      <c r="O33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T33" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996123882583084</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0.969795188277553</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>0.925576196292447</v>
@@ -2924,7 +2348,7 @@
         <v>0.955939758689639</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>0.803793159228948</v>
@@ -2936,40 +2360,22 @@
       <c r="N34" s="3" t="n">
         <v>0.888842583261856</v>
       </c>
-      <c r="O34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S34" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T34" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.998480754546849</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>0.992422611149915</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.980296456463297</v>
@@ -2978,19 +2384,19 @@
         <v>0.99559249838149</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.989772746530277</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>0.927074459274781</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="M35" s="3" t="n">
         <v>0.953409382692888</v>
@@ -2998,34 +2404,16 @@
       <c r="N35" s="3" t="n">
         <v>0.98781745464669</v>
       </c>
-      <c r="O35" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P35" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T35" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.99546884480786</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>0.960943720955395</v>
@@ -3036,7 +2424,7 @@
         <v>0.950982895098882</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>0.773087063383051</v>
@@ -3048,34 +2436,16 @@
       <c r="N36" s="3" t="n">
         <v>0.981035375612377</v>
       </c>
-      <c r="O36" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P36" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T36" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.998932166853944</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0.986810513377358</v>
@@ -3086,19 +2456,19 @@
         <v>0.986570525764206</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>0.936089201810795</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>0.928441807163585</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="M37" s="3" t="n">
         <v>0.986852392055639</v>
@@ -3106,34 +2476,16 @@
       <c r="N37" s="3" t="n">
         <v>0.995222320803457</v>
       </c>
-      <c r="O37" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P37" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T37" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.996905610452122</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0.928329826828612</v>
@@ -3144,7 +2496,7 @@
         <v>0.866109790099055</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>0.645229444653891</v>
@@ -3152,7 +2504,7 @@
       <c r="J38" s="2"/>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0.936729598778588</v>
@@ -3160,34 +2512,16 @@
       <c r="N38" s="3" t="n">
         <v>0.956288683422495</v>
       </c>
-      <c r="O38" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P38" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T38" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.930872311433532</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>0.85041385190883</v>
@@ -3198,7 +2532,7 @@
         <v>0.675995300576774</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>0.746129945546971</v>
@@ -3210,34 +2544,16 @@
       <c r="N39" s="3" t="n">
         <v>0.819795871635397</v>
       </c>
-      <c r="O39" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P39" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T39" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.998465583966881</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>0.995254467848528</v>
@@ -3248,7 +2564,7 @@
         <v>0.997728519333611</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>0.959775759711831</v>
@@ -3256,7 +2572,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0.928952639111837</v>
@@ -3264,34 +2580,16 @@
       <c r="N40" s="3" t="n">
         <v>0.983807389953579</v>
       </c>
-      <c r="O40" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P40" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T40" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.99915778915087</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D41" s="3" t="n">
         <v>0.998585593777231</v>
@@ -3302,7 +2600,7 @@
         <v>0.993154898603039</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>0.941258954609845</v>
@@ -3314,34 +2612,16 @@
       <c r="N41" s="3" t="n">
         <v>0.0573439955343392</v>
       </c>
-      <c r="O41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P41" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T41" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996471867499297</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>0.984695082690026</v>
@@ -3352,7 +2632,7 @@
         <v>0.993773664897899</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>0.559632299427059</v>
@@ -3360,7 +2640,7 @@
       <c r="J42" s="6"/>
       <c r="K42" s="7"/>
       <c r="L42" s="6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="M42" s="7" t="n">
         <v>0.991819220378155</v>
@@ -3368,34 +2648,16 @@
       <c r="N42" s="3" t="n">
         <v>0.557852701797722</v>
       </c>
-      <c r="O42" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P42" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S42" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T42" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.995798184740579</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>0.837689830729731</v>
@@ -3406,7 +2668,7 @@
         <v>0.852573069055459</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>0.289971648819954</v>
@@ -3414,7 +2676,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="7"/>
       <c r="L43" s="6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="M43" s="7" t="n">
         <v>0.991819220378155</v>
@@ -3422,45 +2684,27 @@
       <c r="N43" s="3" t="n">
         <v>0.547301794595584</v>
       </c>
-      <c r="O43" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P43" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R43" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S43" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T43" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>0.669873865803624</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.969213303626853</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.579038811454065</v>
@@ -3470,34 +2714,16 @@
       <c r="L44" s="2"/>
       <c r="M44" s="3"/>
       <c r="N44" s="3"/>
-      <c r="O44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R44" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T44" s="2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.992268993693795</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>0.997904461563255</v>
@@ -3508,7 +2734,7 @@
         <v>0.994479470566958</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>0.504211903569637</v>
@@ -3520,34 +2746,16 @@
       <c r="N45" s="3" t="n">
         <v>0.587167215139279</v>
       </c>
-      <c r="O45" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P45" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q45" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R45" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S45" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T45" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.997445021406782</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>0.994483240276513</v>
@@ -3558,7 +2766,7 @@
         <v>0.976652004477945</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>0.92372504933245</v>
@@ -3570,40 +2778,22 @@
       <c r="N46" s="3" t="n">
         <v>0.0475462843338336</v>
       </c>
-      <c r="O46" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P46" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q46" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R46" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S46" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T46" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>0.963008093248055</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>0.941081172920484</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="F47" s="5" t="n">
         <v>0.937662887460793</v>
@@ -3612,7 +2802,7 @@
         <v>0.968820362778515</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>0.801500318970652</v>
@@ -3624,40 +2814,22 @@
       <c r="N47" s="3" t="n">
         <v>0.102429900117076</v>
       </c>
-      <c r="O47" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P47" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q47" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R47" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S47" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T47" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>0.993313545860852</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D48" s="3" t="n">
         <v>0.983675304699237</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0.909292167040706</v>
@@ -3666,7 +2838,7 @@
         <v>0.963036985482454</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>0.998475150576667</v>
@@ -3678,33 +2850,15 @@
       <c r="N48" s="3" t="n">
         <v>0.986654622703124</v>
       </c>
-      <c r="O48" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P48" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q48" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R48" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="S48" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T48" s="2" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dealing with overview table
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -581,52 +581,52 @@
     <t xml:space="preserve">ID_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 89 Sig ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim vs Type 476 Sig Collapsed to Type 89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linking Tumor ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim vs Linking Tumor Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Best Match to Koh et al., 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim vs Koh et al.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim of Extracted 476-Type Sig vs Linking Tumor Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extracted Type-83 Sig ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim of Extracted 83-Type Sig vs Linking Tumor Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest COSMIC Sig ID to Extracted 83-Type Sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim of COSMIC Sig vs Extracted 83-Type Sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest Sig from Jin et al., 2024 to Extracted 83-Type Sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim of Jin et al. to Extracted 83-Type Sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine Sim vs Type 476 Sig Approx Collapsed to Type 83</t>
+    <t xml:space="preserve">Type 89 Signature ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs&lt;br&gt;Extracted Type 476 Sig&lt;br&gt;Collapsed&lt;br&gt;to Type 89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linking&lt;br&gt;Tumor ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs&lt;br&gt;Linking Tumor&lt;br&gt;Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best Match to&lt;br&gt;Koh et al., 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs&lt;br&gt;Koh et al.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of&lt;br&gt;Extracted 476-Type Sig vs&lt;br&gt;Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extracted&lt;br&gt;Type-83 Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of&lt;br&gt;Extracted 83-Type Sig vs&lt;br&gt;Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest COSMIC Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of&lt;br&gt;COSMIC Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest Sig from&lt;br&gt;Jin et al., 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of&lt;br&gt;Jin et al.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs&lt;br&gt;Type 476 Sig Approx&lt;br&gt;Collapsed to Type 83</t>
   </si>
   <si>
     <t xml:space="preserve">* This is the signature with the best match to the given type-89 signature.</t>
   </si>
   <si>
-    <t xml:space="preserve">** indicates that in the supporting tumor's spectrum, insertions of single Ts in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
+    <t xml:space="preserve">** indicates that in the linking tumor's spectrum, insertions of single Ts in long poly-T contexts were set to 0 before calculating cosine similarity to the 83-type signature.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
working on table 1
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -581,46 +581,46 @@
     <t xml:space="preserve">ID_P</t>
   </si>
   <si>
-    <t xml:space="preserve">Type 89 Signature ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine vs&lt;br&gt;Extracted Type 476 Sig&lt;br&gt;Collapsed&lt;br&gt;to Type 89</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linking&lt;br&gt;Tumor ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine vs&lt;br&gt;Linking Tumor&lt;br&gt;Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Best Match to&lt;br&gt;Koh et al., 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine vs&lt;br&gt;Koh et al.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine of&lt;br&gt;Extracted 476-Type Sig vs&lt;br&gt;Linking Tumor Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extracted&lt;br&gt;Type-83 Sig ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine of&lt;br&gt;Extracted 83-Type Sig vs&lt;br&gt;Linking Tumor Spectrum</t>
+    <t xml:space="preserve">89-Type Classification Signature ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs Extracted 476-Type Sig Collapsed to 89-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linking Tumor ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine 89-Type 89 Sig vs Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best Match to Koh et al., 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine 89-Type Sig vs Koh et al.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of Extracted 476-Type Sig vs Linking Tumor Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extracted 83-Type Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine of Extracted 83-Type Sig vs Linking Tumor Spectrum</t>
   </si>
   <si>
     <t xml:space="preserve">Closest COSMIC Sig ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Cosine of&lt;br&gt;COSMIC Sig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest Sig from&lt;br&gt;Jin et al., 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine of&lt;br&gt;Jin et al.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine vs&lt;br&gt;Type 476 Sig Approx&lt;br&gt;Collapsed to Type 83</t>
+    <t xml:space="preserve">Cosine of COSMIC Sig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closest Sig from Jin et al., 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine vs Jin et al.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine 83-Type vs 476-Type Sig Approx Collapsed to 83-Type</t>
   </si>
   <si>
     <t xml:space="preserve">* This is the signature with the best match to the given type-89 signature.</t>

</xml_diff>

<commit_message>
regenerated vignette html after correcting assgnments; misc file cleanup
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -1443,7 +1443,9 @@
       <c r="A11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3" t="n">
+        <v>0.997924670503285</v>
+      </c>
       <c r="C11" s="2" t="s">
         <v>45</v>
       </c>
@@ -1473,7 +1475,9 @@
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
+      <c r="N11" s="3" t="n">
+        <v>0.939390479737653</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
@@ -1844,7 +1848,7 @@
         <v>88</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.188996059832515</v>
+        <v>0.997918760374102</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>89</v>
@@ -1880,7 +1884,7 @@
         <v>0.983749624551454</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>0.194386082170664</v>
+        <v>0.99354876657351</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
still digging out of the ID16 error due to simple files in 2019
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -327,9 +327,6 @@
   </si>
   <si>
     <t xml:space="preserve">C_ID16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID16</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel17</t>
@@ -1013,46 +1010,46 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="2">
@@ -1140,7 +1137,7 @@
         <v>0.998577618888331</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>0.961637651964785</v>
+        <v>0.961637651964883</v>
       </c>
     </row>
     <row r="4">
@@ -1268,7 +1265,7 @@
         <v>0.998910219006335</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.981397358400931</v>
+        <v>0.981397358400003</v>
       </c>
     </row>
     <row r="7">
@@ -1308,7 +1305,7 @@
         <v>0.998910219006335</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.901007598283463</v>
+        <v>0.901007598283187</v>
       </c>
     </row>
     <row r="8">
@@ -1392,7 +1389,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.913500020598801</v>
+        <v>0.913500021315506</v>
       </c>
     </row>
     <row r="10">
@@ -1436,7 +1433,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.998782441826826</v>
+        <v>0.998782441835448</v>
       </c>
     </row>
     <row r="11">
@@ -1983,29 +1980,23 @@
         <v>104</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="K24" s="3" t="n">
-        <v>0.94431118528519</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J24" s="2"/>
+      <c r="K24" s="3"/>
       <c r="L24" s="2"/>
       <c r="M24" s="3"/>
-      <c r="N24" s="3" t="n">
-        <v>0.672733978429856</v>
-      </c>
+      <c r="N24" s="3"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.999028913454499</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0.999098612098447</v>
@@ -2016,13 +2007,13 @@
         <v>0.999651240340044</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>0.998055396153645</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>0.913211851073001</v>
@@ -2035,19 +2026,19 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.997224063445585</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0.990826011162356</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.997866554870421</v>
@@ -2056,13 +2047,13 @@
         <v>0.983277628405395</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0.926638815378631</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0.9748626883743</v>
@@ -2075,13 +2066,13 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.998016917127346</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0.956199773890916</v>
@@ -2092,13 +2083,13 @@
         <v>0.903787160547224</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.578876004293571</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2111,13 +2102,13 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.998952350407319</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0.991711747199947</v>
@@ -2128,13 +2119,13 @@
         <v>0.982120219990487</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>0.95772281360567</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2147,13 +2138,13 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.997697967449371</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0.59843282958418</v>
@@ -2164,13 +2155,13 @@
         <v>0.567830470268594</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.439321442308408</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2183,13 +2174,13 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.994265618936021</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>0.960618679377363</v>
@@ -2200,13 +2191,13 @@
         <v>0.926005386424851</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>0.966191991161316</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>0.988733344519805</v>
@@ -2219,19 +2210,19 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.997724733557505</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>0.642466773271259</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>0.919336320629207</v>
@@ -2240,7 +2231,7 @@
         <v>0.537837150518689</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.509401386863396</v>
@@ -2259,19 +2250,19 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.993433690246823</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>0.928962481898069</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.965491583372847</v>
@@ -2280,7 +2271,7 @@
         <v>0.937843010334813</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I32" s="7" t="n">
         <v>0.90936321357593</v>
@@ -2299,13 +2290,13 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999703811227718</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>0.985553780930321</v>
@@ -2316,7 +2307,7 @@
         <v>0.971992601692081</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>0.971905124482824</v>
@@ -2331,19 +2322,19 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996123882583084</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0.969795188277553</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>0.925576196292447</v>
@@ -2352,7 +2343,7 @@
         <v>0.955939758689639</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>0.803793159228948</v>
@@ -2367,19 +2358,19 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.998480754546849</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>0.992422611149915</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.980296456463297</v>
@@ -2388,7 +2379,7 @@
         <v>0.99559249838149</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.989772746530277</v>
@@ -2411,13 +2402,13 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.99546884480786</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>0.960943720955395</v>
@@ -2428,7 +2419,7 @@
         <v>0.950982895098882</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>0.773087063383051</v>
@@ -2443,13 +2434,13 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.998932166853944</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0.986810513377358</v>
@@ -2460,7 +2451,7 @@
         <v>0.986570525764206</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>0.936089201810795</v>
@@ -2483,13 +2474,13 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.996905610452122</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0.928329826828612</v>
@@ -2500,7 +2491,7 @@
         <v>0.866109790099055</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>0.645229444653891</v>
@@ -2508,7 +2499,7 @@
       <c r="J38" s="2"/>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0.936729598778588</v>
@@ -2519,13 +2510,13 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.930872311433532</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>0.85041385190883</v>
@@ -2536,7 +2527,7 @@
         <v>0.675995300576774</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>0.746129945546971</v>
@@ -2551,13 +2542,13 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.998465583966881</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>0.995254467848528</v>
@@ -2568,7 +2559,7 @@
         <v>0.997728519333611</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>0.959775759711831</v>
@@ -2576,7 +2567,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0.928952639111837</v>
@@ -2587,13 +2578,13 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.99915778915087</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D41" s="3" t="n">
         <v>0.998585593777231</v>
@@ -2604,7 +2595,7 @@
         <v>0.993154898603039</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>0.941258954609845</v>
@@ -2619,13 +2610,13 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996471867499297</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>0.984695082690026</v>
@@ -2636,7 +2627,7 @@
         <v>0.993773664897899</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>0.559632299427059</v>
@@ -2644,7 +2635,7 @@
       <c r="J42" s="6"/>
       <c r="K42" s="7"/>
       <c r="L42" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M42" s="7" t="n">
         <v>0.991819220378155</v>
@@ -2655,13 +2646,13 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.995798184740579</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>0.837689830729731</v>
@@ -2672,7 +2663,7 @@
         <v>0.852573069055459</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>0.289971648819954</v>
@@ -2680,7 +2671,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="7"/>
       <c r="L43" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M43" s="7" t="n">
         <v>0.991819220378155</v>
@@ -2691,24 +2682,24 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>0.669873865803624</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.969213303626853</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.579038811454065</v>
@@ -2721,13 +2712,13 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.992268993693795</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>0.997904461563255</v>
@@ -2738,7 +2729,7 @@
         <v>0.994479470566958</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>0.504211903569637</v>
@@ -2753,13 +2744,13 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.997445021406782</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>0.994483240276513</v>
@@ -2770,7 +2761,7 @@
         <v>0.976652004477945</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>0.92372504933245</v>
@@ -2785,19 +2776,19 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>0.963008093248055</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>0.941081172920484</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F47" s="5" t="n">
         <v>0.937662887460793</v>
@@ -2806,7 +2797,7 @@
         <v>0.968820362778515</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>0.801500318970652</v>
@@ -2821,19 +2812,19 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>0.993313545860852</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D48" s="3" t="n">
         <v>0.983675304699237</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0.909292167040706</v>
@@ -2842,7 +2833,7 @@
         <v>0.963036985482454</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>0.998475150576667</v>
@@ -2857,12 +2848,12 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add .gitatt... and re-rendered
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -327,6 +327,9 @@
   </si>
   <si>
     <t xml:space="preserve">C_ID16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID16</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel17</t>
@@ -1010,46 +1013,46 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2">
@@ -1181,7 +1184,7 @@
         <v>0.998577618888331</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.995713098771566</v>
+        <v>0.995713098771624</v>
       </c>
     </row>
     <row r="5">
@@ -1389,7 +1392,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.913500021315506</v>
+        <v>0.913500020598801</v>
       </c>
     </row>
     <row r="10">
@@ -1433,7 +1436,7 @@
         <v>0.952591756729311</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.998782441835448</v>
+        <v>0.998782441826826</v>
       </c>
     </row>
     <row r="11">
@@ -1980,23 +1983,29 @@
         <v>104</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2"/>
-      <c r="K24" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="L24" s="2"/>
       <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
+      <c r="N24" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.999028913454499</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0.999098612098447</v>
@@ -2007,13 +2016,13 @@
         <v>0.999651240340044</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>0.998055396153645</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>0.913211851073001</v>
@@ -2026,19 +2035,19 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.997224063445585</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>0.990826011162356</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.997866554870421</v>
@@ -2047,13 +2056,13 @@
         <v>0.983277628405395</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0.926638815378631</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>0.9748626883743</v>
@@ -2066,13 +2075,13 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.998016917127346</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>0.956199773890916</v>
@@ -2083,13 +2092,13 @@
         <v>0.903787160547224</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.578876004293571</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K27" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2102,13 +2111,13 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.998952350407319</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0.991711747199947</v>
@@ -2119,13 +2128,13 @@
         <v>0.982120219990487</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>0.95772281360567</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2138,13 +2147,13 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.997697967449371</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0.59843282958418</v>
@@ -2155,13 +2164,13 @@
         <v>0.567830470268594</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.439321442308408</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>0.934723603717686</v>
@@ -2174,13 +2183,13 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.994265618936021</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>0.960618679377363</v>
@@ -2191,13 +2200,13 @@
         <v>0.926005386424851</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>0.966191991161316</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>0.988733344519805</v>
@@ -2210,19 +2219,19 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.997724733557505</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>0.642466773271259</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>0.919336320629207</v>
@@ -2231,7 +2240,7 @@
         <v>0.537837150518689</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.509401386863396</v>
@@ -2250,19 +2259,19 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.993433690246823</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>0.928962481898069</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.965491583372847</v>
@@ -2271,7 +2280,7 @@
         <v>0.937843010334813</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I32" s="7" t="n">
         <v>0.90936321357593</v>
@@ -2290,13 +2299,13 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999703811227718</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>0.985553780930321</v>
@@ -2307,7 +2316,7 @@
         <v>0.971992601692081</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>0.971905124482824</v>
@@ -2322,19 +2331,19 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996123882583084</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>0.969795188277553</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F34" s="5" t="n">
         <v>0.925576196292447</v>
@@ -2343,7 +2352,7 @@
         <v>0.955939758689639</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>0.803793159228948</v>
@@ -2358,19 +2367,19 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.998480754546849</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>0.992422611149915</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.980296456463297</v>
@@ -2379,7 +2388,7 @@
         <v>0.99559249838149</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.989772746530277</v>
@@ -2402,13 +2411,13 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.99546884480786</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>0.960943720955395</v>
@@ -2419,7 +2428,7 @@
         <v>0.950982895098882</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>0.773087063383051</v>
@@ -2434,13 +2443,13 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.998932166853944</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0.986810513377358</v>
@@ -2451,7 +2460,7 @@
         <v>0.986570525764206</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>0.936089201810795</v>
@@ -2474,13 +2483,13 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.996905610452122</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0.928329826828612</v>
@@ -2491,7 +2500,7 @@
         <v>0.866109790099055</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>0.645229444653891</v>
@@ -2499,7 +2508,7 @@
       <c r="J38" s="2"/>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="M38" s="3" t="n">
         <v>0.936729598778588</v>
@@ -2510,13 +2519,13 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.930872311433532</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>0.85041385190883</v>
@@ -2527,7 +2536,7 @@
         <v>0.675995300576774</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>0.746129945546971</v>
@@ -2542,13 +2551,13 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.998465583966881</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>0.995254467848528</v>
@@ -2559,7 +2568,7 @@
         <v>0.997728519333611</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>0.959775759711831</v>
@@ -2567,7 +2576,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="M40" s="3" t="n">
         <v>0.928952639111837</v>
@@ -2578,13 +2587,13 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.99915778915087</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D41" s="3" t="n">
         <v>0.998585593777231</v>
@@ -2595,7 +2604,7 @@
         <v>0.993154898603039</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>0.941258954609845</v>
@@ -2610,13 +2619,13 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996471867499297</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D42" s="3" t="n">
         <v>0.984695082690026</v>
@@ -2627,7 +2636,7 @@
         <v>0.993773664897899</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I42" s="7" t="n">
         <v>0.559632299427059</v>
@@ -2635,7 +2644,7 @@
       <c r="J42" s="6"/>
       <c r="K42" s="7"/>
       <c r="L42" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M42" s="7" t="n">
         <v>0.991819220378155</v>
@@ -2646,13 +2655,13 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.995798184740579</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>0.837689830729731</v>
@@ -2663,7 +2672,7 @@
         <v>0.852573069055459</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I43" s="7" t="n">
         <v>0.289971648819954</v>
@@ -2671,7 +2680,7 @@
       <c r="J43" s="6"/>
       <c r="K43" s="7"/>
       <c r="L43" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M43" s="7" t="n">
         <v>0.991819220378155</v>
@@ -2682,24 +2691,24 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B44" s="3"/>
       <c r="C44" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>0.669873865803624</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.969213303626853</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I44" s="3" t="n">
         <v>0.579038811454065</v>
@@ -2712,13 +2721,13 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.992268993693795</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D45" s="3" t="n">
         <v>0.997904461563255</v>
@@ -2729,7 +2738,7 @@
         <v>0.994479470566958</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I45" s="3" t="n">
         <v>0.504211903569637</v>
@@ -2744,13 +2753,13 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.997445021406782</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>0.994483240276513</v>
@@ -2761,7 +2770,7 @@
         <v>0.976652004477945</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I46" s="3" t="n">
         <v>0.92372504933245</v>
@@ -2776,19 +2785,19 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B47" s="3" t="n">
         <v>0.963008093248055</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>0.941081172920484</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F47" s="5" t="n">
         <v>0.937662887460793</v>
@@ -2797,7 +2806,7 @@
         <v>0.968820362778515</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I47" s="3" t="n">
         <v>0.801500318970652</v>
@@ -2812,19 +2821,19 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B48" s="3" t="n">
         <v>0.993313545860852</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D48" s="3" t="n">
         <v>0.983675304699237</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F48" s="3" t="n">
         <v>0.909292167040706</v>
@@ -2833,7 +2842,7 @@
         <v>0.963036985482454</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I48" s="3" t="n">
         <v>0.998475150576667</v>
@@ -2848,12 +2857,12 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
still cleaning up vignette
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="232">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">WIDE01010075T</t>
   </si>
   <si>
-    <t xml:space="preserve">SP85864</t>
+    <t xml:space="preserve">SP13539</t>
   </si>
   <si>
     <t xml:space="preserve">InD7</t>
@@ -290,9 +290,6 @@
     <t xml:space="preserve">SP109957</t>
   </si>
   <si>
-    <t xml:space="preserve">SP116919</t>
-  </si>
-  <si>
     <t xml:space="preserve">C_ID10**</t>
   </si>
   <si>
@@ -578,10 +575,7 @@
     <t xml:space="preserve">InsDel_J</t>
   </si>
   <si>
-    <t xml:space="preserve">SP86836</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP85818</t>
+    <t xml:space="preserve">SP112959</t>
   </si>
   <si>
     <t xml:space="preserve">ID_J**</t>
@@ -593,7 +587,7 @@
     <t xml:space="preserve">SP17905</t>
   </si>
   <si>
-    <t xml:space="preserve">SP135192</t>
+    <t xml:space="preserve">SP112257</t>
   </si>
   <si>
     <t xml:space="preserve">InD20</t>
@@ -608,7 +602,7 @@
     <t xml:space="preserve">InsDel_L</t>
   </si>
   <si>
-    <t xml:space="preserve">SP78711</t>
+    <t xml:space="preserve">SP70106</t>
   </si>
   <si>
     <t xml:space="preserve">ID_L</t>
@@ -1104,58 +1098,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="2">
@@ -1897,7 +1891,7 @@
         <v>77</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0.434025442106556</v>
+        <v>0.480808627014228</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.830630961919803</v>
@@ -2037,10 +2031,10 @@
         <v>91</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0.845720420740311</v>
@@ -2048,16 +2042,16 @@
       <c r="G18" s="2"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="n">
-        <v>0.921550902876584</v>
+        <v>0.796363389036035</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>0.796363389036035</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.820516942806174</v>
+        <v>0.752297831081127</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0.752297831081127</v>
@@ -2065,7 +2059,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="3"/>
       <c r="P18" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="Q18" s="3" t="n">
         <v>0.901574092984453</v>
@@ -2076,19 +2070,19 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0.999995205671525</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>0.999995230749744</v>
@@ -2102,7 +2096,7 @@
         <v>0.999999190427207</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>0.998961052288015</v>
@@ -2111,13 +2105,13 @@
         <v>0.998961052288015</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O19" s="3" t="n">
         <v>0.967441621021888</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Q19" s="3" t="n">
         <v>0.997513023097306</v>
@@ -2128,19 +2122,19 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0.990839008275248</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="E20" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0.970118693520178</v>
@@ -2154,7 +2148,7 @@
         <v>0.947101462963348</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L20" s="3" t="n">
         <v>0.957725007713369</v>
@@ -2163,13 +2157,13 @@
         <v>0.740722621050451</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>0.928338601031412</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>0.936826633607344</v>
@@ -2180,25 +2174,25 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0.998943667831344</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="E21" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0.990794529270798</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H21" s="3" t="n">
         <v>0.98860905348304</v>
@@ -2210,7 +2204,7 @@
         <v>0.986008088349909</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>0.991277552948159</v>
@@ -2219,13 +2213,13 @@
         <v>0.989949786954795</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>0.958027843030213</v>
       </c>
       <c r="P21" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q21" s="3" t="n">
         <v>0.958027842856697</v>
@@ -2236,25 +2230,25 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0.997982743475383</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0.994521225549591</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>0.983091970590282</v>
@@ -2266,7 +2260,7 @@
         <v>0.997069663552165</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L22" s="3" t="n">
         <v>0.99651862160547</v>
@@ -2275,13 +2269,13 @@
         <v>0.99651862160547</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O22" s="3" t="n">
         <v>0.932088000143203</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q22" s="3" t="n">
         <v>0.958381270941474</v>
@@ -2292,19 +2286,19 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0.999500630385848</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0.997152554254249</v>
@@ -2318,7 +2312,7 @@
         <v>0.99444026424933</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L23" s="3" t="n">
         <v>0.998116134659162</v>
@@ -2327,7 +2321,7 @@
         <v>0.998116134659162</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="O23" s="3" t="n">
         <v>0.992624379767039</v>
@@ -2344,19 +2338,19 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>1</v>
@@ -2370,7 +2364,7 @@
         <v>1</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L24" s="3" t="n">
         <v>0.983879088998686</v>
@@ -2379,13 +2373,13 @@
         <v>0.0841219391036441</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O24" s="3" t="n">
         <v>0.983749624781302</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>0.983749624640517</v>
@@ -2396,19 +2390,19 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.9999701532808</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>0.999914468437142</v>
@@ -2422,7 +2416,7 @@
         <v>0.999835057995513</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>0.996899575153152</v>
@@ -2431,13 +2425,13 @@
         <v>0.996899575153152</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O25" s="3" t="n">
         <v>0.914053274268444</v>
       </c>
       <c r="P25" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q25" s="3" t="n">
         <v>0.817774909347475</v>
@@ -2448,25 +2442,25 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.99960379787758</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.995835062853617</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>0.995865147542038</v>
@@ -2478,7 +2472,7 @@
         <v>0.985124263787052</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L26" s="3" t="n">
         <v>0.985825843839382</v>
@@ -2487,13 +2481,13 @@
         <v>0.985825843839382</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>0.977804138512642</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Q26" s="3" t="n">
         <v>0.908745880262362</v>
@@ -2504,19 +2498,19 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.991323931809998</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0.949421223719236</v>
@@ -2530,7 +2524,7 @@
         <v>0.842103236395361</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L27" s="7" t="n">
         <v>0.989493745287417</v>
@@ -2541,7 +2535,7 @@
       <c r="N27" s="6"/>
       <c r="O27" s="7"/>
       <c r="P27" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q27" s="7" t="n">
         <v>0.77303146395448</v>
@@ -2552,19 +2546,19 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.996336204909843</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0.992203974046295</v>
@@ -2578,7 +2572,7 @@
         <v>0.974928977461464</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L28" s="7" t="n">
         <v>0.989493745287417</v>
@@ -2589,7 +2583,7 @@
       <c r="N28" s="6"/>
       <c r="O28" s="7"/>
       <c r="P28" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q28" s="7" t="n">
         <v>0.77303146395448</v>
@@ -2600,19 +2594,19 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.914042638364057</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0.826204117287774</v>
@@ -2626,7 +2620,7 @@
         <v>0.531769407979438</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L29" s="7" t="n">
         <v>0.989493745287417</v>
@@ -2637,7 +2631,7 @@
       <c r="N29" s="6"/>
       <c r="O29" s="7"/>
       <c r="P29" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q29" s="7" t="n">
         <v>0.77303146395448</v>
@@ -2648,19 +2642,19 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.970093629514313</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>0.960574846051305</v>
@@ -2674,7 +2668,7 @@
         <v>0.909235484677089</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L30" s="3" t="n">
         <v>0.966402041939997</v>
@@ -2683,7 +2677,7 @@
         <v>0.966402041939997</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O30" s="3" t="n">
         <v>0.988648649042165</v>
@@ -2700,19 +2694,19 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.998172880224683</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="E31" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0.809677297354619</v>
@@ -2726,7 +2720,7 @@
         <v>0.767562040163278</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="L31" s="7" t="n">
         <v>0.822699200845167</v>
@@ -2748,25 +2742,25 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.992666731131994</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.936066841399292</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>0.965031393647406</v>
@@ -2778,7 +2772,7 @@
         <v>0.939987653380814</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="L32" s="7" t="n">
         <v>0.822699200845167</v>
@@ -2800,19 +2794,19 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999911654065824</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="E33" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0.987166551488096</v>
@@ -2826,7 +2820,7 @@
         <v>0.974893777989085</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L33" s="3" t="n">
         <v>0.992425785100674</v>
@@ -2848,25 +2842,25 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996791829608519</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0.971347929143106</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H34" s="5" t="n">
         <v>0.92677979381067</v>
@@ -2878,7 +2872,7 @@
         <v>0.958339841652829</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>0.826745670634646</v>
@@ -2889,7 +2883,7 @@
       <c r="N34" s="2"/>
       <c r="O34" s="3"/>
       <c r="P34" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Q34" s="3" t="n">
         <v>0.550967765579797</v>
@@ -2900,25 +2894,25 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.999639620152708</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="E35" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.999921059710238</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>0.925706920608922</v>
@@ -2930,7 +2924,7 @@
         <v>0.999743108117304</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L35" s="3" t="n">
         <v>0.959840394712428</v>
@@ -2952,19 +2946,19 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.998357669632125</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="E36" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0.97761298883184</v>
@@ -2978,7 +2972,7 @@
         <v>0.951583104137893</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L36" s="3" t="n">
         <v>0.898847174499529</v>
@@ -2989,7 +2983,7 @@
       <c r="N36" s="2"/>
       <c r="O36" s="3"/>
       <c r="P36" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q36" s="3" t="n">
         <v>0.818969949993968</v>
@@ -3000,19 +2994,19 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.999335497592149</v>
       </c>
       <c r="C37" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="E37" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0.992503948290037</v>
@@ -3026,7 +3020,7 @@
         <v>0.989916400630042</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="L37" s="3" t="n">
         <v>0.968303600199824</v>
@@ -3037,7 +3031,7 @@
       <c r="N37" s="2"/>
       <c r="O37" s="3"/>
       <c r="P37" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q37" s="3" t="n">
         <v>0.972597475832869</v>
@@ -3048,19 +3042,19 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.998026282136621</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0.954658409385147</v>
@@ -3074,7 +3068,7 @@
         <v>0.905800423526931</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L38" s="3" t="n">
         <v>0.732165024027759</v>
@@ -3085,7 +3079,7 @@
       <c r="N38" s="2"/>
       <c r="O38" s="3"/>
       <c r="P38" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="Q38" s="3" t="n">
         <v>0.946706660713885</v>
@@ -3096,19 +3090,19 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.973160707237346</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0.820571179855277</v>
@@ -3122,7 +3116,7 @@
         <v>0.679103818816574</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L39" s="3" t="n">
         <v>0.814121696361617</v>
@@ -3144,19 +3138,19 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.99905266647622</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>0.99977300427146</v>
@@ -3170,7 +3164,7 @@
         <v>0.997679042336974</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L40" s="3" t="n">
         <v>0.967598279961637</v>
@@ -3181,7 +3175,7 @@
       <c r="N40" s="2"/>
       <c r="O40" s="3"/>
       <c r="P40" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Q40" s="3" t="n">
         <v>0.932320876680087</v>
@@ -3192,44 +3186,44 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.975340835478923</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.882497479723799</v>
+        <v>0.717737931500204</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3" t="n">
-        <v>0.9545435686468</v>
+        <v>0.740483106030332</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.936215686347334</v>
+        <v>0.740483106030332</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>0.895000244023661</v>
+        <v>0.73484576506459</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.895000244023661</v>
+        <v>0.73484576506459</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="3"/>
       <c r="P41" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q41" s="3" t="n">
         <v>0.759882547340309</v>
@@ -3240,25 +3234,25 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996358428040646</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0.857208955423799</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H42" s="3" t="n">
         <v>0.910682893126815</v>
@@ -3270,10 +3264,10 @@
         <v>0.857836026177924</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>0.625315741819866</v>
+        <v>0.567227490814057</v>
       </c>
       <c r="M42" s="3" t="n">
         <v>0.270321860201427</v>
@@ -3281,7 +3275,7 @@
       <c r="N42" s="2"/>
       <c r="O42" s="3"/>
       <c r="P42" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="Q42" s="3" t="n">
         <v>0.981466622733605</v>
@@ -3292,19 +3286,19 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.998096980390783</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0.965794892044298</v>
@@ -3318,10 +3312,10 @@
         <v>0.940623718327597</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.695434384162641</v>
+        <v>0.58696107449826</v>
       </c>
       <c r="M43" s="3" t="n">
         <v>0.275022162638091</v>
@@ -3329,7 +3323,7 @@
       <c r="N43" s="2"/>
       <c r="O43" s="3"/>
       <c r="P43" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="Q43" s="3" t="n">
         <v>0.86996795258408</v>
@@ -3340,19 +3334,19 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B44" s="3" t="n">
         <v>0.999833476696041</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>85</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.999915018177657</v>
@@ -3366,7 +3360,7 @@
         <v>0.999668997798308</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L44" s="3" t="n">
         <v>0.719554188496143</v>
@@ -3388,25 +3382,25 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.989972335380856</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>0.984044585558769</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>0.922936622532135</v>
@@ -3418,7 +3412,7 @@
         <v>0.949717052461629</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L45" s="7" t="n">
         <v>0.0799102187135878</v>
@@ -3440,25 +3434,25 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.987932278009431</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>0.986631173660937</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>0.917332176399582</v>
@@ -3470,7 +3464,7 @@
         <v>0.958852538451186</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="L46" s="7" t="n">
         <v>0.0799102187135878</v>
@@ -3492,12 +3486,12 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
got up to date spectra for the tcga sample with ID16
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="233">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -86,6 +86,9 @@
     <t xml:space="preserve">ID1</t>
   </si>
   <si>
+    <t xml:space="preserve">ID1*</t>
+  </si>
+  <si>
     <t xml:space="preserve">InsDel1b</t>
   </si>
   <si>
@@ -128,6 +131,9 @@
     <t xml:space="preserve">ID2</t>
   </si>
   <si>
+    <t xml:space="preserve">ID2*</t>
+  </si>
+  <si>
     <t xml:space="preserve">InsDel2b</t>
   </si>
   <si>
@@ -155,6 +161,9 @@
     <t xml:space="preserve">ID3</t>
   </si>
   <si>
+    <t xml:space="preserve">ID3*</t>
+  </si>
+  <si>
     <t xml:space="preserve">InsDel3b</t>
   </si>
   <si>
@@ -179,9 +188,6 @@
     <t xml:space="preserve">C_ID4</t>
   </si>
   <si>
-    <t xml:space="preserve">ID24</t>
-  </si>
-  <si>
     <t xml:space="preserve">InsDel5a</t>
   </si>
   <si>
@@ -281,9 +287,6 @@
     <t xml:space="preserve">C_ID9</t>
   </si>
   <si>
-    <t xml:space="preserve">ID9</t>
-  </si>
-  <si>
     <t xml:space="preserve">InsDel10</t>
   </si>
   <si>
@@ -383,6 +386,9 @@
     <t xml:space="preserve">C_ID16</t>
   </si>
   <si>
+    <t xml:space="preserve">ID13*</t>
+  </si>
+  <si>
     <t xml:space="preserve">InsDel17</t>
   </si>
   <si>
@@ -425,36 +431,36 @@
     <t xml:space="preserve">C_ID19</t>
   </si>
   <si>
+    <t xml:space="preserve">InsDel19b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02050192T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02340081T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02020734T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02340026T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID23</t>
+  </si>
+  <si>
     <t xml:space="preserve">ID23</t>
   </si>
   <si>
-    <t xml:space="preserve">InsDel19b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02050192T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340081T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02020734T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340026T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID23</t>
-  </si>
-  <si>
     <t xml:space="preserve">InsDel_A_alpha</t>
   </si>
   <si>
@@ -524,54 +530,54 @@
     <t xml:space="preserve">ID_E</t>
   </si>
   <si>
+    <t xml:space="preserve">InsDel_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01030028T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP5559</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01030015T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02010648T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP107439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_I</t>
+  </si>
+  <si>
     <t xml:space="preserve">ID25</t>
   </si>
   <si>
-    <t xml:space="preserve">InsDel_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01030028T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP5559</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01030015T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID11b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010648T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP107439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_I</t>
-  </si>
-  <si>
     <t xml:space="preserve">InsDel_J</t>
   </si>
   <si>
@@ -606,9 +612,6 @@
   </si>
   <si>
     <t xml:space="preserve">ID_L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID20</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel_M</t>
@@ -714,9 +717,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -763,7 +767,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -780,10 +784,19 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1098,58 +1111,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2">
@@ -1183,25 +1196,25 @@
       <c r="J2" s="3" t="n">
         <v>0.955622755229959</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="7" t="n">
+      <c r="L2" s="8" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M2" s="7" t="n">
+      <c r="M2" s="8" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="7" t="n">
+      <c r="O2" s="8" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" s="7" t="n">
+      <c r="P2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q2" s="8" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R2" s="3" t="n">
@@ -1210,25 +1223,25 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.995751609987239</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.984963988162326</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>0.979574035620553</v>
@@ -1239,25 +1252,25 @@
       <c r="J3" s="3" t="n">
         <v>0.983594266371644</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="7" t="n">
+      <c r="L3" s="8" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M3" s="7" t="n">
+      <c r="M3" s="8" t="n">
         <v>0.984693782257925</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="8" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="7" t="n">
+      <c r="Q3" s="10" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R3" s="3" t="n">
@@ -1266,25 +1279,25 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.972816786949883</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.967513714073498</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0.941518994163211</v>
@@ -1295,25 +1308,25 @@
       <c r="J4" s="3" t="n">
         <v>0.922180889933715</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="7" t="n">
+      <c r="L4" s="8" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M4" s="7" t="n">
+      <c r="M4" s="8" t="n">
         <v>0.991458286142515</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="7" t="n">
+      <c r="O4" s="8" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="P4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" s="7" t="n">
+      <c r="Q4" s="10" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R4" s="3" t="n">
@@ -1322,25 +1335,25 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.975888181735629</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0.969793210503792</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>0.942250946766091</v>
@@ -1351,25 +1364,25 @@
       <c r="J5" s="3" t="n">
         <v>0.945783579633834</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" s="7" t="n">
+      <c r="K5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="8" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M5" s="7" t="n">
+      <c r="M5" s="8" t="n">
         <v>0.962198073105692</v>
       </c>
-      <c r="N5" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" s="7" t="n">
+      <c r="N5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" s="8" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P5" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" s="7" t="n">
+      <c r="P5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="8" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R5" s="3" t="n">
@@ -1378,19 +1391,19 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.985774863204943</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0.964494916249486</v>
@@ -1403,25 +1416,25 @@
       <c r="J6" s="3" t="n">
         <v>0.965908193462833</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L6" s="7" t="n">
+      <c r="K6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" s="8" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M6" s="7" t="n">
+      <c r="M6" s="8" t="n">
         <v>0.985731547816123</v>
       </c>
-      <c r="N6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="O6" s="7" t="n">
+      <c r="N6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" s="8" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q6" s="7" t="n">
+      <c r="P6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" s="10" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R6" s="3" t="n">
@@ -1430,19 +1443,19 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.984219619129365</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0.974439597022551</v>
@@ -1455,25 +1468,25 @@
       <c r="J7" s="3" t="n">
         <v>0.98546887561434</v>
       </c>
-      <c r="K7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L7" s="7" t="n">
+      <c r="K7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" s="8" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M7" s="7" t="n">
+      <c r="M7" s="8" t="n">
         <v>0.990258473144984</v>
       </c>
-      <c r="N7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="O7" s="7" t="n">
+      <c r="N7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7" s="8" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q7" s="7" t="n">
+      <c r="P7" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q7" s="10" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R7" s="3" t="n">
@@ -1482,19 +1495,19 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0.991203953894052</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0.973836073095472</v>
@@ -1507,25 +1520,25 @@
       <c r="J8" s="3" t="n">
         <v>0.913578014108215</v>
       </c>
-      <c r="K8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="L8" s="7" t="n">
+      <c r="K8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L8" s="8" t="n">
         <v>0.997300319860517</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="M8" s="8" t="n">
         <v>0.847828402800451</v>
       </c>
-      <c r="N8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O8" s="7" t="n">
+      <c r="N8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="O8" s="8" t="n">
         <v>0.985685429503426</v>
       </c>
-      <c r="P8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q8" s="7" t="n">
+      <c r="P8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q8" s="8" t="n">
         <v>0.940287785159075</v>
       </c>
       <c r="R8" s="3" t="n">
@@ -1534,25 +1547,25 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.999045131608235</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0.995211832270212</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>0.952660131778202</v>
@@ -1563,25 +1576,25 @@
       <c r="J9" s="3" t="n">
         <v>0.988850250718193</v>
       </c>
-      <c r="K9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="L9" s="7" t="n">
+      <c r="K9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L9" s="8" t="n">
         <v>0.997300319860517</v>
       </c>
-      <c r="M9" s="7" t="n">
+      <c r="M9" s="8" t="n">
         <v>0.997112251828433</v>
       </c>
-      <c r="N9" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O9" s="7" t="n">
+      <c r="N9" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="O9" s="8" t="n">
         <v>0.985685429503426</v>
       </c>
-      <c r="P9" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q9" s="7" t="n">
+      <c r="P9" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q9" s="10" t="n">
         <v>0.940287785159075</v>
       </c>
       <c r="R9" s="3" t="n">
@@ -1590,25 +1603,25 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.995469513052381</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0.984487609245987</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>0.982035840377093</v>
@@ -1620,7 +1633,7 @@
         <v>0.944193811816217</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>0.985571290231238</v>
@@ -1630,37 +1643,33 @@
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="3"/>
-      <c r="P10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>0.79333762252597</v>
-      </c>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="3"/>
       <c r="R10" s="3" t="n">
         <v>0.930675294514924</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>0.999948468759238</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.99077239403383</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>0.948827781549115</v>
@@ -1671,46 +1680,42 @@
       <c r="J11" s="3" t="n">
         <v>0.975851323620917</v>
       </c>
-      <c r="K11" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="L11" s="7" t="n">
+      <c r="K11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="L11" s="8" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M11" s="7" t="n">
+      <c r="M11" s="8" t="n">
         <v>0.991027893423615</v>
       </c>
-      <c r="N11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="O11" s="7" t="n">
+      <c r="N11" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="O11" s="8" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q11" s="7" t="n">
-        <v>0.896852917912874</v>
-      </c>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="8"/>
       <c r="R11" s="3" t="n">
         <v>0.999825580341641</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0.995334597849054</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0.982577764855043</v>
@@ -1723,46 +1728,42 @@
       <c r="J12" s="3" t="n">
         <v>0.944499430908083</v>
       </c>
-      <c r="K12" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="L12" s="7" t="n">
+      <c r="K12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M12" s="7" t="n">
+      <c r="M12" s="8" t="n">
         <v>0.711038761231236</v>
       </c>
-      <c r="N12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="O12" s="7" t="n">
+      <c r="N12" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q12" s="7" t="n">
-        <v>0.896852917912874</v>
-      </c>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="8"/>
       <c r="R12" s="3" t="n">
         <v>0.771635129733512</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>0.97793690362112</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>0.934392717811593</v>
@@ -1775,52 +1776,48 @@
       <c r="J13" s="3" t="n">
         <v>0.872318581377061</v>
       </c>
-      <c r="K13" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="L13" s="7" t="n">
+      <c r="K13" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="8" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M13" s="7" t="n">
+      <c r="M13" s="8" t="n">
         <v>0.542517905062245</v>
       </c>
-      <c r="N13" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="O13" s="7" t="n">
+      <c r="N13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="O13" s="8" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P13" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q13" s="7" t="n">
-        <v>0.896852917912874</v>
-      </c>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="8"/>
       <c r="R13" s="3" t="n">
         <v>0.679463517454566</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>0.998146874520311</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0.994938158549685</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0.974493620999996</v>
@@ -1832,7 +1829,7 @@
         <v>0.991460194711972</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>0.995324626236781</v>
@@ -1841,13 +1838,13 @@
         <v>0.992535120953994</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0.957398848117212</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="Q14" s="3" t="n">
         <v>0.915585976377244</v>
@@ -1858,25 +1855,25 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>0.997720161516685</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0.996684575409509</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>0.979743628092745</v>
@@ -1888,7 +1885,7 @@
         <v>0.995235008498556</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>0.480808627014228</v>
@@ -1897,42 +1894,38 @@
         <v>0.830630961919803</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O15" s="3" t="n">
         <v>0.954696316779994</v>
       </c>
-      <c r="P15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q15" s="3" t="n">
-        <v>0.892827491603587</v>
-      </c>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="3"/>
       <c r="R15" s="3" t="n">
         <v>0.124136591318613</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0.994244367584137</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0.991418420361293</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>0.981178677303978</v>
@@ -1944,7 +1937,7 @@
         <v>0.997890073647472</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>0.970244652019643</v>
@@ -1953,13 +1946,13 @@
         <v>0.970244652019643</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0.988370367422066</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Q16" s="3" t="n">
         <v>0.968325984027352</v>
@@ -1970,25 +1963,25 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>0.999233924465169</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0.925869318345882</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>0.916987691583686</v>
@@ -2000,7 +1993,7 @@
         <v>0.792129011416151</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L17" s="3" t="n">
         <v>0.948672768843191</v>
@@ -2010,31 +2003,27 @@
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="3"/>
-      <c r="P17" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>0.763790768753592</v>
-      </c>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="3"/>
       <c r="R17" s="3" t="n">
         <v>0.998318979193059</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0.956900109132159</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0.845720420740311</v>
@@ -2048,7 +2037,7 @@
         <v>0.796363389036035</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>0.752297831081127</v>
@@ -2059,7 +2048,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="3"/>
       <c r="P18" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q18" s="3" t="n">
         <v>0.901574092984453</v>
@@ -2070,19 +2059,19 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0.999995205671525</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>0.999995230749744</v>
@@ -2096,7 +2085,7 @@
         <v>0.999999190427207</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>0.998961052288015</v>
@@ -2105,13 +2094,13 @@
         <v>0.998961052288015</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O19" s="3" t="n">
         <v>0.967441621021888</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q19" s="3" t="n">
         <v>0.997513023097306</v>
@@ -2122,19 +2111,19 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0.990839008275248</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D20" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0.970118693520178</v>
@@ -2148,7 +2137,7 @@
         <v>0.947101462963348</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L20" s="3" t="n">
         <v>0.957725007713369</v>
@@ -2157,13 +2146,13 @@
         <v>0.740722621050451</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>0.928338601031412</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>0.936826633607344</v>
@@ -2174,25 +2163,25 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0.998943667831344</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0.990794529270798</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H21" s="3" t="n">
         <v>0.98860905348304</v>
@@ -2204,7 +2193,7 @@
         <v>0.986008088349909</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>0.991277552948159</v>
@@ -2213,15 +2202,15 @@
         <v>0.989949786954795</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>0.958027843030213</v>
       </c>
-      <c r="P21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q21" s="3" t="n">
+      <c r="P21" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q21" s="6" t="n">
         <v>0.958027842856697</v>
       </c>
       <c r="R21" s="3" t="n">
@@ -2230,25 +2219,25 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0.997982743475383</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0.994521225549591</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>0.983091970590282</v>
@@ -2260,7 +2249,7 @@
         <v>0.997069663552165</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L22" s="3" t="n">
         <v>0.99651862160547</v>
@@ -2269,13 +2258,13 @@
         <v>0.99651862160547</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="O22" s="3" t="n">
         <v>0.932088000143203</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q22" s="3" t="n">
         <v>0.958381270941474</v>
@@ -2286,19 +2275,19 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0.999500630385848</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0.997152554254249</v>
@@ -2312,7 +2301,7 @@
         <v>0.99444026424933</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L23" s="3" t="n">
         <v>0.998116134659162</v>
@@ -2321,36 +2310,32 @@
         <v>0.998116134659162</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O23" s="3" t="n">
         <v>0.992624379767039</v>
       </c>
-      <c r="P23" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q23" s="3" t="n">
-        <v>0.700155777261457</v>
-      </c>
+      <c r="P23" s="2"/>
+      <c r="Q23" s="3"/>
       <c r="R23" s="3" t="n">
         <v>0.999700940744567</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>1</v>
@@ -2364,7 +2349,7 @@
         <v>1</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L24" s="3" t="n">
         <v>0.983879088998686</v>
@@ -2373,13 +2358,13 @@
         <v>0.0841219391036441</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O24" s="3" t="n">
         <v>0.983749624781302</v>
       </c>
       <c r="P24" s="2" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>0.983749624640517</v>
@@ -2390,19 +2375,19 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.9999701532808</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>0.999914468437142</v>
@@ -2416,7 +2401,7 @@
         <v>0.999835057995513</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>0.996899575153152</v>
@@ -2425,42 +2410,38 @@
         <v>0.996899575153152</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="O25" s="3" t="n">
         <v>0.914053274268444</v>
       </c>
-      <c r="P25" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q25" s="3" t="n">
-        <v>0.817774909347475</v>
-      </c>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="3"/>
       <c r="R25" s="3" t="n">
         <v>0.997931218812211</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>0.99960379787758</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.995835062853617</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>0.995865147542038</v>
@@ -2472,7 +2453,7 @@
         <v>0.985124263787052</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L26" s="3" t="n">
         <v>0.985825843839382</v>
@@ -2481,13 +2462,13 @@
         <v>0.985825843839382</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>0.977804138512642</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="Q26" s="3" t="n">
         <v>0.908745880262362</v>
@@ -2498,19 +2479,19 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.991323931809998</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0.949421223719236</v>
@@ -2523,42 +2504,38 @@
       <c r="J27" s="3" t="n">
         <v>0.842103236395361</v>
       </c>
-      <c r="K27" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="L27" s="7" t="n">
+      <c r="K27" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L27" s="8" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M27" s="7" t="n">
+      <c r="M27" s="8" t="n">
         <v>0.54831345887048</v>
       </c>
-      <c r="N27" s="6"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="Q27" s="7" t="n">
-        <v>0.77303146395448</v>
-      </c>
+      <c r="N27" s="7"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="8"/>
       <c r="R27" s="3" t="n">
         <v>0.725714494601862</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0.996336204909843</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0.992203974046295</v>
@@ -2571,42 +2548,38 @@
       <c r="J28" s="3" t="n">
         <v>0.974928977461464</v>
       </c>
-      <c r="K28" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="L28" s="7" t="n">
+      <c r="K28" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L28" s="8" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M28" s="7" t="n">
+      <c r="M28" s="8" t="n">
         <v>0.985557763846102</v>
       </c>
-      <c r="N28" s="6"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="Q28" s="7" t="n">
-        <v>0.77303146395448</v>
-      </c>
+      <c r="N28" s="7"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="7"/>
+      <c r="Q28" s="8"/>
       <c r="R28" s="3" t="n">
         <v>0.989653793004506</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.914042638364057</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0.826204117287774</v>
@@ -2619,42 +2592,38 @@
       <c r="J29" s="3" t="n">
         <v>0.531769407979438</v>
       </c>
-      <c r="K29" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="L29" s="7" t="n">
+      <c r="K29" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="L29" s="8" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M29" s="7" t="n">
+      <c r="M29" s="8" t="n">
         <v>0.502264030394843</v>
       </c>
-      <c r="N29" s="6"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="Q29" s="7" t="n">
-        <v>0.77303146395448</v>
-      </c>
+      <c r="N29" s="7"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="7"/>
+      <c r="Q29" s="8"/>
       <c r="R29" s="3" t="n">
         <v>0.855443301955089</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0.970093629514313</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>0.960574846051305</v>
@@ -2668,7 +2637,7 @@
         <v>0.909235484677089</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L30" s="3" t="n">
         <v>0.966402041939997</v>
@@ -2677,36 +2646,32 @@
         <v>0.966402041939997</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="O30" s="3" t="n">
         <v>0.988648649042165</v>
       </c>
-      <c r="P30" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q30" s="3" t="n">
-        <v>0.729410321267104</v>
-      </c>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="3"/>
       <c r="R30" s="3" t="n">
         <v>0.970130472042864</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0.998172880224683</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0.809677297354619</v>
@@ -2719,48 +2684,44 @@
       <c r="J31" s="3" t="n">
         <v>0.767562040163278</v>
       </c>
-      <c r="K31" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="L31" s="7" t="n">
+      <c r="K31" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="L31" s="8" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="M31" s="7" t="n">
+      <c r="M31" s="8" t="n">
         <v>0.433810499900094</v>
       </c>
-      <c r="N31" s="6"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q31" s="7" t="n">
-        <v>0.890460217074095</v>
-      </c>
+      <c r="N31" s="7"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="7"/>
+      <c r="Q31" s="8"/>
       <c r="R31" s="3" t="n">
         <v>0.962491763279905</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0.992666731131994</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.936066841399292</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>0.965031393647406</v>
@@ -2771,42 +2732,38 @@
       <c r="J32" s="3" t="n">
         <v>0.939987653380814</v>
       </c>
-      <c r="K32" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="L32" s="7" t="n">
+      <c r="K32" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="L32" s="8" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="M32" s="7" t="n">
+      <c r="M32" s="8" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="N32" s="6"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q32" s="7" t="n">
-        <v>0.890460217074095</v>
-      </c>
+      <c r="N32" s="7"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="7"/>
+      <c r="Q32" s="8"/>
       <c r="R32" s="3" t="n">
         <v>0.894656202812139</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0.999911654065824</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0.987166551488096</v>
@@ -2820,7 +2777,7 @@
         <v>0.974893777989085</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L33" s="3" t="n">
         <v>0.992425785100674</v>
@@ -2830,37 +2787,33 @@
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="3"/>
-      <c r="P33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q33" s="3" t="n">
-        <v>0.676931318353377</v>
-      </c>
+      <c r="P33" s="2"/>
+      <c r="Q33" s="3"/>
       <c r="R33" s="3" t="n">
         <v>0.64276888240939</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996791829608519</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0.971347929143106</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H34" s="5" t="n">
         <v>0.92677979381067</v>
@@ -2872,7 +2825,7 @@
         <v>0.958339841652829</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>0.826745670634646</v>
@@ -2882,37 +2835,33 @@
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="3"/>
-      <c r="P34" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q34" s="3" t="n">
-        <v>0.550967765579797</v>
-      </c>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="3"/>
       <c r="R34" s="3" t="n">
         <v>0.88776388540597</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0.999639620152708</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>0.999921059710238</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>0.925706920608922</v>
@@ -2924,7 +2873,7 @@
         <v>0.999743108117304</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="L35" s="3" t="n">
         <v>0.959840394712428</v>
@@ -2934,31 +2883,27 @@
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="3"/>
-      <c r="P35" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q35" s="3" t="n">
-        <v>0.728792755594034</v>
-      </c>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="3"/>
       <c r="R35" s="3" t="n">
         <v>0.838276765666799</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0.998357669632125</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0.97761298883184</v>
@@ -2972,7 +2917,7 @@
         <v>0.951583104137893</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="L36" s="3" t="n">
         <v>0.898847174499529</v>
@@ -2982,31 +2927,27 @@
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="3"/>
-      <c r="P36" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q36" s="3" t="n">
-        <v>0.818969949993968</v>
-      </c>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="3"/>
       <c r="R36" s="3" t="n">
         <v>0.953146317599159</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.999335497592149</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D37" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>172</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0.992503948290037</v>
@@ -3020,7 +2961,7 @@
         <v>0.989916400630042</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L37" s="3" t="n">
         <v>0.968303600199824</v>
@@ -3031,7 +2972,7 @@
       <c r="N37" s="2"/>
       <c r="O37" s="3"/>
       <c r="P37" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q37" s="3" t="n">
         <v>0.972597475832869</v>
@@ -3042,19 +2983,19 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0.998026282136621</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0.954658409385147</v>
@@ -3068,7 +3009,7 @@
         <v>0.905800423526931</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L38" s="3" t="n">
         <v>0.732165024027759</v>
@@ -3079,7 +3020,7 @@
       <c r="N38" s="2"/>
       <c r="O38" s="3"/>
       <c r="P38" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q38" s="3" t="n">
         <v>0.946706660713885</v>
@@ -3090,19 +3031,19 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0.973160707237346</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0.820571179855277</v>
@@ -3116,7 +3057,7 @@
         <v>0.679103818816574</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L39" s="3" t="n">
         <v>0.814121696361617</v>
@@ -3126,31 +3067,27 @@
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="3"/>
-      <c r="P39" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q39" s="3" t="n">
-        <v>0.622520949750488</v>
-      </c>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="3"/>
       <c r="R39" s="3" t="n">
         <v>0.812996997625178</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.99905266647622</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>0.99977300427146</v>
@@ -3164,7 +3101,7 @@
         <v>0.997679042336974</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="L40" s="3" t="n">
         <v>0.967598279961637</v>
@@ -3175,7 +3112,7 @@
       <c r="N40" s="2"/>
       <c r="O40" s="3"/>
       <c r="P40" s="2" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="Q40" s="3" t="n">
         <v>0.932320876680087</v>
@@ -3186,19 +3123,19 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.975340835478923</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0.717737931500204</v>
@@ -3212,7 +3149,7 @@
         <v>0.740483106030332</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="L41" s="3" t="n">
         <v>0.73484576506459</v>
@@ -3222,37 +3159,33 @@
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="3"/>
-      <c r="P41" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="Q41" s="3" t="n">
-        <v>0.759882547340309</v>
-      </c>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="3"/>
       <c r="R41" s="3" t="n">
         <v>0.817490469929235</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996358428040646</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0.857208955423799</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H42" s="3" t="n">
         <v>0.910682893126815</v>
@@ -3264,7 +3197,7 @@
         <v>0.857836026177924</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="L42" s="3" t="n">
         <v>0.567227490814057</v>
@@ -3275,7 +3208,7 @@
       <c r="N42" s="2"/>
       <c r="O42" s="3"/>
       <c r="P42" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="Q42" s="3" t="n">
         <v>0.981466622733605</v>
@@ -3286,19 +3219,19 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.998096980390783</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0.965794892044298</v>
@@ -3312,7 +3245,7 @@
         <v>0.940623718327597</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="L43" s="3" t="n">
         <v>0.58696107449826</v>
@@ -3322,31 +3255,27 @@
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="3"/>
-      <c r="P43" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q43" s="3" t="n">
-        <v>0.86996795258408</v>
-      </c>
+      <c r="P43" s="2"/>
+      <c r="Q43" s="3"/>
       <c r="R43" s="3" t="n">
         <v>0.491570915468926</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B44" s="3" t="n">
         <v>0.999833476696041</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.999915018177657</v>
@@ -3360,7 +3289,7 @@
         <v>0.999668997798308</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="L44" s="3" t="n">
         <v>0.719554188496143</v>
@@ -3370,37 +3299,33 @@
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="3"/>
-      <c r="P44" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q44" s="3" t="n">
-        <v>0.668558358110025</v>
-      </c>
+      <c r="P44" s="2"/>
+      <c r="Q44" s="3"/>
       <c r="R44" s="3" t="n">
         <v>0.722798931979844</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.989972335380856</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>0.984044585558769</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>0.922936622532135</v>
@@ -3411,48 +3336,44 @@
       <c r="J45" s="3" t="n">
         <v>0.949717052461629</v>
       </c>
-      <c r="K45" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="L45" s="7" t="n">
+      <c r="K45" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="L45" s="8" t="n">
         <v>0.0799102187135878</v>
       </c>
-      <c r="M45" s="7" t="n">
+      <c r="M45" s="8" t="n">
         <v>0.0596010478033871</v>
       </c>
-      <c r="N45" s="6"/>
-      <c r="O45" s="7"/>
-      <c r="P45" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>0.79226521622831</v>
-      </c>
+      <c r="N45" s="7"/>
+      <c r="O45" s="8"/>
+      <c r="P45" s="7"/>
+      <c r="Q45" s="8"/>
       <c r="R45" s="3" t="n">
         <v>0.982449966334136</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B46" s="3" t="n">
         <v>0.987932278009431</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>0.986631173660937</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>0.917332176399582</v>
@@ -3463,35 +3384,31 @@
       <c r="J46" s="3" t="n">
         <v>0.958852538451186</v>
       </c>
-      <c r="K46" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="L46" s="7" t="n">
+      <c r="K46" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="L46" s="8" t="n">
         <v>0.0799102187135878</v>
       </c>
-      <c r="M46" s="7" t="n">
+      <c r="M46" s="8" t="n">
         <v>0.0783023694574505</v>
       </c>
-      <c r="N46" s="6"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>0.79226521622831</v>
-      </c>
+      <c r="N46" s="7"/>
+      <c r="O46" s="8"/>
+      <c r="P46" s="7"/>
+      <c r="Q46" s="8"/>
       <c r="R46" s="3" t="n">
         <v>0.98410266953065</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
much improved; need to check vhelpers line 246+ calculating residual
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -71,543 +71,555 @@
     <t xml:space="preserve">InsDel1a</t>
   </si>
   <si>
+    <t xml:space="preserve">CPCT02050439T</t>
+  </si>
+  <si>
     <t xml:space="preserve">SP107784</t>
   </si>
   <si>
-    <t xml:space="preserve">CPCT02010523T</t>
+    <t xml:space="preserve">InD14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID1*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP21400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP16886</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel1c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112907</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP125809</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD14*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP17172</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01080031T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02011050T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD2a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID2*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP96118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel2c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01330020T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02050436T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02020815T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02040317T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID3*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02080086T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP48008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP23925</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD4a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel5a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP97194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102755</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel5b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112290</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel5c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP8564</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP28659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP67609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WIDE01010075T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP13539</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID7**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02070336T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102617</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP116520</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD9b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP109957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID10**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP77956</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112947</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02060291T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02050424T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD13*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02340014T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02050104T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WES::TCGA-EW-A2FV-01A-11D-A17D-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WES::TCGA-13-0889-01A-01W-0420-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02250003T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02070053T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02010408TII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02080139T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02010408T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02050192T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02340081T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel19c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02020734T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02340026T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_ID23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_A_alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02120078T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP2293</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_A_beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD9a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02020413T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP116578</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02010772T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02100101T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP116834</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP102133</t>
   </si>
   <si>
     <t xml:space="preserve">InD1</t>
   </si>
   <si>
-    <t xml:space="preserve">C_ID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID1*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel1b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP21400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel1c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112907</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02050439T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010955T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01080031T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02030277T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD2b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID2*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP96118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel2c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01330020T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02050436T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02020815T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID3*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel3b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02080086T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD3b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP48008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP23925</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD4a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel5a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP97194</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102755</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel5b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112290</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel5c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP8564</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP59803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP67609</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WIDE01010075T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP13539</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID7**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02070336T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP116520</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD9b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP109957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID10**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP77956</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID11a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112947</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112985</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02060291T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02050424T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD13*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340014T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WES::TCGA-EW-A2FV-01A-11D-A17D-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WES::TCGA-13-0889-01A-01W-0420-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP124319</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID13*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02250003T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02070053T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010408TII</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02080139T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010408T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02050192T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340081T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel19c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02020734T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340026T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102957</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_ID23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_A_alpha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02120078T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP2293</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_A_beta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD9a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02020413T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112182</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010772T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP102133</t>
+    <t xml:space="preserve">ID_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01340014T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01340015T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01030028T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP5559</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRUP01030015T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID11b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPCT02010648T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP107439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112959</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_J**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP17905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP112257</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InD20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID_K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InsDel_L</t>
   </si>
   <si>
     <t xml:space="preserve">CPCT02450014T</t>
   </si>
   <si>
-    <t xml:space="preserve">InD19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01340014T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01340015T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01030028T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP5559</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRUP01030015T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID11b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02010648T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP107439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112959</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_J**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP17905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP112257</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID_K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InsDel_L</t>
-  </si>
-  <si>
     <t xml:space="preserve">SP70106</t>
   </si>
   <si>
@@ -644,13 +656,7 @@
     <t xml:space="preserve">InsDel_N_beta</t>
   </si>
   <si>
-    <t xml:space="preserve">SP111031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02210064T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InD2a</t>
+    <t xml:space="preserve">InD21</t>
   </si>
   <si>
     <t xml:space="preserve">89-Type Classification Signature ID</t>
@@ -767,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -782,9 +788,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1111,58 +1114,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2">
@@ -1170,55 +1173,55 @@
         <v>18</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.994633203355323</v>
+        <v>0.99225514421935</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="F2" s="3" t="n">
-        <v>0.981145366226036</v>
-      </c>
-      <c r="G2" s="2" t="s">
+        <v>0.983074166010633</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>0.923732254214595</v>
+      <c r="H2" s="5" t="n">
+        <v>0.902299689128411</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.96004253323919</v>
+        <v>0.977133136425943</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.955622755229959</v>
-      </c>
-      <c r="K2" s="7" t="s">
+        <v>0.977133136425943</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="8" t="n">
+      <c r="L2" s="7" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M2" s="8" t="n">
-        <v>0.998618143772308</v>
-      </c>
-      <c r="N2" s="7" t="s">
+      <c r="M2" s="7" t="n">
+        <v>0.995814528115091</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="8" t="n">
+      <c r="O2" s="7" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Q2" s="8" t="n">
+      <c r="Q2" s="7" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.996710141979561</v>
+        <v>0.996541760045853</v>
       </c>
     </row>
     <row r="3">
@@ -1226,184 +1229,184 @@
         <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.995751609987239</v>
+        <v>0.992510031716818</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.984963988162326</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>0.979574035620553</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.983594266371644</v>
+        <v>0.97139996588332</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.983594266371644</v>
-      </c>
-      <c r="K3" s="7" t="s">
+        <v>0.970117181733333</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="8" t="n">
+      <c r="L3" s="7" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M3" s="8" t="n">
+      <c r="M3" s="7" t="n">
         <v>0.984693782257925</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="8" t="n">
+      <c r="O3" s="7" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Q3" s="10" t="n">
+      <c r="Q3" s="9" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>0.991554867288987</v>
+        <v>0.991662053669514</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.972816786949883</v>
+        <v>0.981866350977739</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>0.967513714073498</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>0.941518994163211</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.979918877112646</v>
+        <v>0.908213126613381</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.922180889933715</v>
-      </c>
-      <c r="K4" s="7" t="s">
+        <v>0.900924066128503</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="L4" s="7" t="n">
         <v>0.998618143772308</v>
       </c>
-      <c r="M4" s="8" t="n">
+      <c r="M4" s="7" t="n">
         <v>0.991458286142515</v>
       </c>
-      <c r="N4" s="7" t="s">
+      <c r="N4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="8" t="n">
+      <c r="O4" s="7" t="n">
         <v>0.98452971866307</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Q4" s="10" t="n">
+      <c r="Q4" s="9" t="n">
         <v>0.984922448705973</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.989228469487461</v>
+        <v>0.99630805359721</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.975888181735629</v>
+        <v>0.985294543813336</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.969793210503792</v>
+        <v>0.971029412068895</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.942250946766091</v>
+        <v>0.982386171804305</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.959033747752441</v>
+        <v>0.980234171516011</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.945783579633834</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5" s="8" t="n">
+        <v>0.972607282708758</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L5" s="7" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M5" s="8" t="n">
-        <v>0.962198073105692</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="O5" s="8" t="n">
+      <c r="M5" s="7" t="n">
+        <v>0.998590592344902</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="7" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q5" s="8" t="n">
+      <c r="P5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q5" s="7" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.992615020267686</v>
+        <v>0.999377186450455</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.985774863204943</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>0.964494916249486</v>
@@ -1416,25 +1419,25 @@
       <c r="J6" s="3" t="n">
         <v>0.965908193462833</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L6" s="8" t="n">
+      <c r="K6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="7" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="M6" s="7" t="n">
         <v>0.985731547816123</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="O6" s="8" t="n">
+      <c r="N6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" s="7" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P6" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q6" s="10" t="n">
+      <c r="P6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" s="9" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R6" s="3" t="n">
@@ -1443,19 +1446,19 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.984219619129365</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0.974439597022551</v>
@@ -1468,25 +1471,25 @@
       <c r="J7" s="3" t="n">
         <v>0.98546887561434</v>
       </c>
-      <c r="K7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" s="8" t="n">
+      <c r="K7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="7" t="n">
         <v>0.999575040995962</v>
       </c>
-      <c r="M7" s="8" t="n">
+      <c r="M7" s="7" t="n">
         <v>0.990258473144984</v>
       </c>
-      <c r="N7" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="O7" s="8" t="n">
+      <c r="N7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O7" s="7" t="n">
         <v>0.979933784936098</v>
       </c>
-      <c r="P7" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q7" s="10" t="n">
+      <c r="P7" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" s="9" t="n">
         <v>0.993151664730949</v>
       </c>
       <c r="R7" s="3" t="n">
@@ -1495,19 +1498,19 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.991203953894052</v>
+        <v>0.951485153830059</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0.973836073095472</v>
@@ -1515,113 +1518,113 @@
       <c r="G8" s="2"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3" t="n">
-        <v>0.913578014108215</v>
+        <v>0.939627373336213</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.913578014108215</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="L8" s="8" t="n">
+        <v>0.804482903759715</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="7" t="n">
         <v>0.997300319860517</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="M8" s="7" t="n">
         <v>0.847828402800451</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="O8" s="8" t="n">
+      <c r="N8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="O8" s="7" t="n">
         <v>0.985685429503426</v>
       </c>
-      <c r="P8" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q8" s="8" t="n">
+      <c r="P8" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q8" s="7" t="n">
         <v>0.940287785159075</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.926000159889564</v>
+        <v>0.945396131140755</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.999045131608235</v>
+        <v>0.996989110119111</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0.995211832270212</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>0.952660131778202</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.993408206018199</v>
+        <v>0.992475624937649</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.988850250718193</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="L9" s="8" t="n">
+        <v>0.98366871012917</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="L9" s="7" t="n">
         <v>0.997300319860517</v>
       </c>
-      <c r="M9" s="8" t="n">
+      <c r="M9" s="7" t="n">
         <v>0.997112251828433</v>
       </c>
-      <c r="N9" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="O9" s="8" t="n">
+      <c r="N9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="O9" s="7" t="n">
         <v>0.985685429503426</v>
       </c>
-      <c r="P9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q9" s="10" t="n">
+      <c r="P9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q9" s="9" t="n">
         <v>0.940287785159075</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0.999816160931316</v>
+        <v>0.995424708706045</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.995469513052381</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0.984487609245987</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>0.982035840377093</v>
@@ -1633,7 +1636,7 @@
         <v>0.944193811816217</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>0.985571290231238</v>
@@ -1651,71 +1654,71 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.999948468759238</v>
+        <v>0.998300408496317</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.99077239403383</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>0.948827781549115</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.975851323620917</v>
+        <v>0.971762010175488</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.975851323620917</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="L11" s="8" t="n">
+        <v>0.971762010175488</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="L11" s="7" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M11" s="8" t="n">
+      <c r="M11" s="7" t="n">
         <v>0.991027893423615</v>
       </c>
-      <c r="N11" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="O11" s="8" t="n">
+      <c r="N11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="O11" s="7" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="8"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="7"/>
       <c r="R11" s="3" t="n">
-        <v>0.999825580341641</v>
+        <v>0.997684298092557</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0.995334597849054</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0.982577764855043</v>
@@ -1728,42 +1731,42 @@
       <c r="J12" s="3" t="n">
         <v>0.944499430908083</v>
       </c>
-      <c r="K12" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="L12" s="8" t="n">
+      <c r="K12" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="L12" s="7" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M12" s="8" t="n">
+      <c r="M12" s="7" t="n">
         <v>0.711038761231236</v>
       </c>
-      <c r="N12" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="O12" s="8" t="n">
+      <c r="N12" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="O12" s="7" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="8"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="7"/>
       <c r="R12" s="3" t="n">
         <v>0.771635129733512</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.97793690362112</v>
+        <v>0.957464756373615</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>0.934392717811593</v>
@@ -1771,53 +1774,53 @@
       <c r="G13" s="2"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="n">
-        <v>0.892792987560485</v>
+        <v>0.907751106430914</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.872318581377061</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="L13" s="8" t="n">
+        <v>0.847252237949434</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="L13" s="7" t="n">
         <v>0.994799526477391</v>
       </c>
-      <c r="M13" s="8" t="n">
+      <c r="M13" s="7" t="n">
         <v>0.542517905062245</v>
       </c>
-      <c r="N13" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="O13" s="8" t="n">
+      <c r="N13" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="O13" s="7" t="n">
         <v>0.908667984436548</v>
       </c>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="8"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="7"/>
       <c r="R13" s="3" t="n">
-        <v>0.679463517454566</v>
+        <v>0.841022969900306</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>0.998146874520311</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>0.994938158549685</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0.974493620999996</v>
@@ -1829,7 +1832,7 @@
         <v>0.991460194711972</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>0.995324626236781</v>
@@ -1838,13 +1841,13 @@
         <v>0.992535120953994</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0.957398848117212</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q14" s="3" t="n">
         <v>0.915585976377244</v>
@@ -1855,25 +1858,25 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>0.997720161516685</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0.996684575409509</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>0.979743628092745</v>
@@ -1885,7 +1888,7 @@
         <v>0.995235008498556</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>0.480808627014228</v>
@@ -1894,7 +1897,7 @@
         <v>0.830630961919803</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O15" s="3" t="n">
         <v>0.954696316779994</v>
@@ -1907,25 +1910,25 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0.994244367584137</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0.991418420361293</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>0.981178677303978</v>
@@ -1937,7 +1940,7 @@
         <v>0.997890073647472</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>0.970244652019643</v>
@@ -1946,13 +1949,13 @@
         <v>0.970244652019643</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0.988370367422066</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="Q16" s="3" t="n">
         <v>0.968325984027352</v>
@@ -1963,25 +1966,25 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>0.999233924465169</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>0.925869318345882</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>0.916987691583686</v>
@@ -1993,7 +1996,7 @@
         <v>0.792129011416151</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="L17" s="3" t="n">
         <v>0.948672768843191</v>
@@ -2011,19 +2014,19 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0.956900109132159</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>0.845720420740311</v>
@@ -2037,7 +2040,7 @@
         <v>0.796363389036035</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>0.752297831081127</v>
@@ -2048,7 +2051,7 @@
       <c r="N18" s="2"/>
       <c r="O18" s="3"/>
       <c r="P18" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Q18" s="3" t="n">
         <v>0.901574092984453</v>
@@ -2059,19 +2062,19 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.999995205671525</v>
+        <v>0.999980561635366</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>0.999995230749744</v>
@@ -2079,13 +2082,13 @@
       <c r="G19" s="2"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="n">
-        <v>0.999999190427207</v>
+        <v>0.999851336466042</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.999999190427207</v>
+        <v>0.999851336466042</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L19" s="3" t="n">
         <v>0.998961052288015</v>
@@ -2094,36 +2097,36 @@
         <v>0.998961052288015</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="O19" s="3" t="n">
         <v>0.967441621021888</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="Q19" s="3" t="n">
         <v>0.997513023097306</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>0.999058367897031</v>
+        <v>0.999408423329615</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0.990839008275248</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0.970118693520178</v>
@@ -2137,7 +2140,7 @@
         <v>0.947101462963348</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L20" s="3" t="n">
         <v>0.957725007713369</v>
@@ -2146,13 +2149,13 @@
         <v>0.740722621050451</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>0.928338601031412</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>0.936826633607344</v>
@@ -2163,37 +2166,37 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.998943667831344</v>
+        <v>0.996183366092605</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0.990794529270798</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H21" s="3" t="n">
         <v>0.98860905348304</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.991649121340236</v>
+        <v>0.995274203111051</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.986008088349909</v>
+        <v>0.98197936808871</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>0.991277552948159</v>
@@ -2202,54 +2205,54 @@
         <v>0.989949786954795</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>0.958027843030213</v>
       </c>
-      <c r="P21" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q21" s="6" t="n">
+      <c r="P21" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q21" s="3" t="n">
         <v>0.958027842856697</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>0.999127035942973</v>
+        <v>0.995953612024326</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.997982743475383</v>
+        <v>0.988147728174671</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0.994521225549591</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>0.983091970590282</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0.997069663552165</v>
+        <v>0.983947390156569</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.997069663552165</v>
+        <v>0.977530389103557</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L22" s="3" t="n">
         <v>0.99651862160547</v>
@@ -2258,36 +2261,36 @@
         <v>0.99651862160547</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O22" s="3" t="n">
         <v>0.932088000143203</v>
       </c>
       <c r="P22" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="Q22" s="3" t="n">
         <v>0.958381270941474</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.999624253509056</v>
+        <v>0.985527676131329</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.999500630385848</v>
+        <v>0.999977796574874</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0.997152554254249</v>
@@ -2295,13 +2298,13 @@
       <c r="G23" s="2"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3" t="n">
-        <v>0.99444026424933</v>
+        <v>0.99471604325606</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.99444026424933</v>
+        <v>0.99471604325606</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="L23" s="3" t="n">
         <v>0.998116134659162</v>
@@ -2310,7 +2313,7 @@
         <v>0.998116134659162</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="O23" s="3" t="n">
         <v>0.992624379767039</v>
@@ -2318,24 +2321,24 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="3"/>
       <c r="R23" s="3" t="n">
-        <v>0.999700940744567</v>
+        <v>0.99998950928761</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F24" s="3" t="n">
         <v>1</v>
@@ -2349,45 +2352,41 @@
         <v>1</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.983879088998686</v>
+        <v>1</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.0841219391036441</v>
+        <v>1</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.983749624781302</v>
-      </c>
-      <c r="P24" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q24" s="3" t="n">
-        <v>0.983749624640517</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="3"/>
       <c r="R24" s="3" t="n">
-        <v>0.101178655678357</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0.9999701532808</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>0.999914468437142</v>
@@ -2401,7 +2400,7 @@
         <v>0.999835057995513</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>0.996899575153152</v>
@@ -2410,7 +2409,7 @@
         <v>0.996899575153152</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="O25" s="3" t="n">
         <v>0.914053274268444</v>
@@ -2423,37 +2422,37 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.99960379787758</v>
+        <v>0.999368087482014</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>0.995835062853617</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>0.995865147542038</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0.985124263787052</v>
+        <v>0.986804557824535</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.985124263787052</v>
+        <v>0.986804557824535</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="L26" s="3" t="n">
         <v>0.985825843839382</v>
@@ -2462,36 +2461,36 @@
         <v>0.985825843839382</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>0.977804138512642</v>
       </c>
       <c r="P26" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="Q26" s="3" t="n">
         <v>0.908745880262362</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>0.999174062469296</v>
+        <v>0.998820438844383</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>0.991323931809998</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0.949421223719236</v>
@@ -2504,38 +2503,38 @@
       <c r="J27" s="3" t="n">
         <v>0.842103236395361</v>
       </c>
-      <c r="K27" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="L27" s="8" t="n">
+      <c r="K27" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="L27" s="7" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M27" s="8" t="n">
+      <c r="M27" s="7" t="n">
         <v>0.54831345887048</v>
       </c>
-      <c r="N27" s="7"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="8"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="7"/>
       <c r="R27" s="3" t="n">
         <v>0.725714494601862</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.996336204909843</v>
+        <v>0.994265744437547</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>0.992203974046295</v>
@@ -2543,43 +2542,43 @@
       <c r="G28" s="2"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3" t="n">
-        <v>0.982941595554607</v>
+        <v>0.986756134212349</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.974928977461464</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="L28" s="8" t="n">
+        <v>0.969862426621788</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="L28" s="7" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M28" s="8" t="n">
+      <c r="M28" s="7" t="n">
         <v>0.985557763846102</v>
       </c>
-      <c r="N28" s="7"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="8"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="7"/>
       <c r="R28" s="3" t="n">
-        <v>0.989653793004506</v>
+        <v>0.998426211868732</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0.914042638364057</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F29" s="3" t="n">
         <v>0.826204117287774</v>
@@ -2592,38 +2591,38 @@
       <c r="J29" s="3" t="n">
         <v>0.531769407979438</v>
       </c>
-      <c r="K29" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="L29" s="8" t="n">
+      <c r="K29" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="L29" s="7" t="n">
         <v>0.989493745287417</v>
       </c>
-      <c r="M29" s="8" t="n">
+      <c r="M29" s="7" t="n">
         <v>0.502264030394843</v>
       </c>
-      <c r="N29" s="7"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="8"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="7"/>
       <c r="R29" s="3" t="n">
         <v>0.855443301955089</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>0.970093629514313</v>
+        <v>0.994537951503423</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>0.960574846051305</v>
@@ -2631,13 +2630,13 @@
       <c r="G30" s="2"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3" t="n">
-        <v>0.909235484677089</v>
+        <v>0.926005384982305</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.909235484677089</v>
+        <v>0.926005384982305</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L30" s="3" t="n">
         <v>0.966402041939997</v>
@@ -2646,7 +2645,7 @@
         <v>0.966402041939997</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="O30" s="3" t="n">
         <v>0.988648649042165</v>
@@ -2654,24 +2653,24 @@
       <c r="P30" s="2"/>
       <c r="Q30" s="3"/>
       <c r="R30" s="3" t="n">
-        <v>0.970130472042864</v>
+        <v>0.990553845591206</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B31" s="3" t="n">
-        <v>0.998172880224683</v>
+        <v>0.997211211367285</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>0.809677297354619</v>
@@ -2679,91 +2678,91 @@
       <c r="G31" s="2"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3" t="n">
-        <v>0.767562040163278</v>
+        <v>0.763564613951013</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>0.767562040163278</v>
-      </c>
-      <c r="K31" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="L31" s="8" t="n">
+        <v>0.763564613951013</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="L31" s="7" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="M31" s="8" t="n">
+      <c r="M31" s="7" t="n">
         <v>0.433810499900094</v>
       </c>
-      <c r="N31" s="7"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="8"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="7"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="7"/>
       <c r="R31" s="3" t="n">
-        <v>0.962491763279905</v>
+        <v>0.959733407276896</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.979201582661447</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B32" s="3" t="n">
-        <v>0.992666731131994</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>0.936066841399292</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>0.965031393647406</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>0.939987653380814</v>
+        <v>0.942020841668772</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.939987653380814</v>
-      </c>
-      <c r="K32" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="L32" s="8" t="n">
+        <v>0.942020841668772</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="L32" s="7" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="M32" s="8" t="n">
+      <c r="M32" s="7" t="n">
         <v>0.822699200845167</v>
       </c>
-      <c r="N32" s="7"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="8"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="7"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="7"/>
       <c r="R32" s="3" t="n">
-        <v>0.894656202812139</v>
+        <v>0.895414993154444</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.999911654065824</v>
+        <v>0.991946464271282</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>0.987166551488096</v>
@@ -2771,49 +2770,49 @@
       <c r="G33" s="2"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3" t="n">
-        <v>0.974893777989085</v>
+        <v>0.971914959592856</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.974893777989085</v>
+        <v>0.971914959592856</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.992425785100674</v>
+        <v>0.983005770605164</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.73143724105477</v>
+        <v>0.965867188155843</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="3"/>
       <c r="P33" s="2"/>
       <c r="Q33" s="3"/>
       <c r="R33" s="3" t="n">
-        <v>0.64276888240939</v>
+        <v>0.981685023255263</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0.996791829608519</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>0.971347929143106</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H34" s="5" t="n">
         <v>0.92677979381067</v>
@@ -2825,7 +2824,7 @@
         <v>0.958339841652829</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>0.826745670634646</v>
@@ -2843,67 +2842,67 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0.999639620152708</v>
+        <v>0.974631943814364</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0.999921059710238</v>
+        <v>0.98789098096416</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>0.925706920608922</v>
+        <v>0.925648389884552</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>0.999743108117304</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.999743108117304</v>
+        <v>0.958707592156772</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>0.959840394712428</v>
+        <v>0.431295771654927</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.838931492257372</v>
+        <v>0.160797754844287</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="3"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="3" t="n">
-        <v>0.838276765666799</v>
+        <v>0.163224677420419</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.998357669632125</v>
+        <v>0.987889331039285</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0.97761298883184</v>
@@ -2911,13 +2910,13 @@
       <c r="G36" s="2"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3" t="n">
-        <v>0.951583104137893</v>
+        <v>0.937108256523303</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.951583104137893</v>
+        <v>0.937108256523303</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="L36" s="3" t="n">
         <v>0.898847174499529</v>
@@ -2930,24 +2929,24 @@
       <c r="P36" s="2"/>
       <c r="Q36" s="3"/>
       <c r="R36" s="3" t="n">
-        <v>0.953146317599159</v>
+        <v>0.974928376963719</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0.999335497592149</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0.992503948290037</v>
@@ -2961,7 +2960,7 @@
         <v>0.989916400630042</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="L37" s="3" t="n">
         <v>0.968303600199824</v>
@@ -2972,7 +2971,7 @@
       <c r="N37" s="2"/>
       <c r="O37" s="3"/>
       <c r="P37" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="Q37" s="3" t="n">
         <v>0.972597475832869</v>
@@ -2983,19 +2982,19 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>0.998026282136621</v>
+        <v>0.996609000779965</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>0.954658409385147</v>
@@ -3003,13 +3002,13 @@
       <c r="G38" s="2"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3" t="n">
-        <v>0.905800423526931</v>
+        <v>0.895518879742724</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.905800423526931</v>
+        <v>0.895518879742724</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="L38" s="3" t="n">
         <v>0.732165024027759</v>
@@ -3020,30 +3019,30 @@
       <c r="N38" s="2"/>
       <c r="O38" s="3"/>
       <c r="P38" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Q38" s="3" t="n">
         <v>0.946706660713885</v>
       </c>
       <c r="R38" s="3" t="n">
-        <v>0.925566903575784</v>
+        <v>0.940849790973729</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.973160707237346</v>
+        <v>0.953973626393374</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>0.820571179855277</v>
@@ -3051,13 +3050,13 @@
       <c r="G39" s="2"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3" t="n">
-        <v>0.679103818816574</v>
+        <v>0.691459114038687</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.679103818816574</v>
+        <v>0.691459114038687</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="L39" s="3" t="n">
         <v>0.814121696361617</v>
@@ -3070,24 +3069,24 @@
       <c r="P39" s="2"/>
       <c r="Q39" s="3"/>
       <c r="R39" s="3" t="n">
-        <v>0.812996997625178</v>
+        <v>0.819606277788974</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0.99905266647622</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>0.99977300427146</v>
@@ -3101,7 +3100,7 @@
         <v>0.997679042336974</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="L40" s="3" t="n">
         <v>0.967598279961637</v>
@@ -3112,7 +3111,7 @@
       <c r="N40" s="2"/>
       <c r="O40" s="3"/>
       <c r="P40" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="Q40" s="3" t="n">
         <v>0.932320876680087</v>
@@ -3123,19 +3122,19 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0.975340835478923</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>0.717737931500204</v>
@@ -3149,7 +3148,7 @@
         <v>0.740483106030332</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="L41" s="3" t="n">
         <v>0.73484576506459</v>
@@ -3167,25 +3166,25 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0.996358428040646</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0.857208955423799</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H42" s="3" t="n">
         <v>0.910682893126815</v>
@@ -3197,7 +3196,7 @@
         <v>0.857836026177924</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="L42" s="3" t="n">
         <v>0.567227490814057</v>
@@ -3208,7 +3207,7 @@
       <c r="N42" s="2"/>
       <c r="O42" s="3"/>
       <c r="P42" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="Q42" s="3" t="n">
         <v>0.981466622733605</v>
@@ -3219,19 +3218,19 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0.998096980390783</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>165</v>
+        <v>201</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>165</v>
+        <v>201</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>0.965794892044298</v>
@@ -3245,7 +3244,7 @@
         <v>0.940623718327597</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="L43" s="3" t="n">
         <v>0.58696107449826</v>
@@ -3263,19 +3262,19 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>0.999833476696041</v>
+        <v>0.994235749511032</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F44" s="3" t="n">
         <v>0.999915018177657</v>
@@ -3283,13 +3282,13 @@
       <c r="G44" s="2"/>
       <c r="H44" s="3"/>
       <c r="I44" s="3" t="n">
-        <v>0.999668997798308</v>
+        <v>0.994583527351464</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.999668997798308</v>
+        <v>0.994583527351464</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="L44" s="3" t="n">
         <v>0.719554188496143</v>
@@ -3302,30 +3301,30 @@
       <c r="P44" s="2"/>
       <c r="Q44" s="3"/>
       <c r="R44" s="3" t="n">
-        <v>0.722798931979844</v>
+        <v>0.788182601795223</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0.989972335380856</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F45" s="3" t="n">
         <v>0.984044585558769</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>0.922936622532135</v>
@@ -3336,79 +3335,79 @@
       <c r="J45" s="3" t="n">
         <v>0.949717052461629</v>
       </c>
-      <c r="K45" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="L45" s="8" t="n">
+      <c r="K45" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="L45" s="7" t="n">
         <v>0.0799102187135878</v>
       </c>
-      <c r="M45" s="8" t="n">
+      <c r="M45" s="7" t="n">
         <v>0.0596010478033871</v>
       </c>
-      <c r="N45" s="7"/>
-      <c r="O45" s="8"/>
-      <c r="P45" s="7"/>
-      <c r="Q45" s="8"/>
+      <c r="N45" s="6"/>
+      <c r="O45" s="7"/>
+      <c r="P45" s="6"/>
+      <c r="Q45" s="7"/>
       <c r="R45" s="3" t="n">
         <v>0.982449966334136</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0.994871170695365</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B46" s="3" t="n">
-        <v>0.987932278009431</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>210</v>
-      </c>
       <c r="D46" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>0.986631173660937</v>
+        <v>0.984978168635262</v>
       </c>
       <c r="G46" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0.904679325987352</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0.967306958360872</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0.967306958360872</v>
+      </c>
+      <c r="K46" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H46" s="3" t="n">
-        <v>0.917332176399582</v>
-      </c>
-      <c r="I46" s="3" t="n">
-        <v>0.976976811437406</v>
-      </c>
-      <c r="J46" s="3" t="n">
-        <v>0.958852538451186</v>
-      </c>
-      <c r="K46" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="L46" s="8" t="n">
+      <c r="L46" s="7" t="n">
         <v>0.0799102187135878</v>
       </c>
-      <c r="M46" s="8" t="n">
-        <v>0.0783023694574505</v>
-      </c>
-      <c r="N46" s="7"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="7"/>
-      <c r="Q46" s="8"/>
+      <c r="M46" s="7" t="n">
+        <v>0.0799102187135878</v>
+      </c>
+      <c r="N46" s="6"/>
+      <c r="O46" s="7"/>
+      <c r="P46" s="6"/>
+      <c r="Q46" s="7"/>
       <c r="R46" s="3" t="n">
-        <v>0.98410266953065</v>
+        <v>0.998239644693817</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-rendered w alt params for residu; edits to prot table xlsx
</commit_message>
<xml_diff>
--- a/vignette/prot_table_1.xlsx
+++ b/vignette/prot_table_1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="233">
   <si>
     <t xml:space="preserve">signature_id</t>
   </si>
@@ -446,15 +446,6 @@
     <t xml:space="preserve">CPCT02340081T</t>
   </si>
   <si>
-    <t xml:space="preserve">InsDel19c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02020734T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPCT02340026T</t>
-  </si>
-  <si>
     <t xml:space="preserve">InsDel23</t>
   </si>
   <si>
@@ -590,6 +581,9 @@
     <t xml:space="preserve">InsDel_J</t>
   </si>
   <si>
+    <t xml:space="preserve">DRUP01010037T</t>
+  </si>
+  <si>
     <t xml:space="preserve">SP112959</t>
   </si>
   <si>
@@ -650,7 +644,7 @@
     <t xml:space="preserve">InD16b</t>
   </si>
   <si>
-    <t xml:space="preserve">ID_N**</t>
+    <t xml:space="preserve">ID_N</t>
   </si>
   <si>
     <t xml:space="preserve">InsDel_N_beta</t>
@@ -1114,58 +1108,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2">
@@ -1173,7 +1167,7 @@
         <v>18</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.99225514421935</v>
+        <v>0.992255142965221</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>19</v>
@@ -1185,43 +1179,43 @@
         <v>19</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.983074166010633</v>
+        <v>0.983074166206997</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>0.902299689128411</v>
+        <v>0.902299690593055</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.977133136425943</v>
+        <v>0.977133137680596</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.977133136425943</v>
+        <v>0.977133137680596</v>
       </c>
       <c r="K2" s="6" t="s">
         <v>22</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>0.998618143772308</v>
+        <v>0.9986181437895</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>0.995814528115091</v>
+        <v>0.995814528097991</v>
       </c>
       <c r="N2" s="6" t="s">
         <v>23</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>0.98452971866307</v>
+        <v>0.984529718633037</v>
       </c>
       <c r="P2" s="6" t="s">
         <v>24</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>0.984922448705973</v>
+        <v>0.984922448681081</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.996541760045853</v>
+        <v>0.996541759404099</v>
       </c>
     </row>
     <row r="3">
@@ -1229,7 +1223,7 @@
         <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>0.992510031716818</v>
+        <v>0.992510044644143</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
@@ -1241,43 +1235,43 @@
         <v>27</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.984963988162326</v>
+        <v>0.984963987993242</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>28</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.979574035620553</v>
+        <v>0.979574035881082</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.97139996588332</v>
+        <v>0.971399962918932</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.970117181733333</v>
+        <v>0.970117178871699</v>
       </c>
       <c r="K3" s="6" t="s">
         <v>22</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>0.998618143772308</v>
+        <v>0.9986181437895</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>0.984693782257925</v>
+        <v>0.984693782178287</v>
       </c>
       <c r="N3" s="6" t="s">
         <v>23</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>0.98452971866307</v>
+        <v>0.984529718633037</v>
       </c>
       <c r="P3" s="8" t="s">
         <v>23</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>0.984922448705973</v>
+        <v>0.984922448681081</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>0.991662053669514</v>
+        <v>0.991662052937842</v>
       </c>
     </row>
     <row r="4">
@@ -1285,7 +1279,7 @@
         <v>29</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.981866350977739</v>
+        <v>0.981866375036531</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>30</v>
@@ -1297,43 +1291,43 @@
         <v>31</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.967513714073498</v>
+        <v>0.967513714201868</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>32</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.941518994163211</v>
+        <v>0.941518994814764</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.908213126613381</v>
+        <v>0.90821311843689</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.900924066128503</v>
+        <v>0.900924071642789</v>
       </c>
       <c r="K4" s="6" t="s">
         <v>22</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>0.998618143772308</v>
+        <v>0.9986181437895</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>0.991458286142515</v>
+        <v>0.991458286236991</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>0.98452971866307</v>
+        <v>0.984529718633037</v>
       </c>
       <c r="P4" s="8" t="s">
         <v>23</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>0.984922448705973</v>
+        <v>0.984922448681081</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.99630805359721</v>
+        <v>0.996308050590285</v>
       </c>
     </row>
     <row r="5">
@@ -1341,7 +1335,7 @@
         <v>33</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0.985294543813336</v>
+        <v>0.985294551259857</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>34</v>
@@ -1353,43 +1347,43 @@
         <v>36</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.971029412068895</v>
+        <v>0.971029412189185</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>37</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.982386171804305</v>
+        <v>0.982386172138281</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.980234171516011</v>
+        <v>0.980234172421836</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.972607282708758</v>
+        <v>0.972607281712882</v>
       </c>
       <c r="K5" s="6" t="s">
         <v>38</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>0.999575040995962</v>
+        <v>0.999575040979855</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>0.998590592344902</v>
+        <v>0.998590592341524</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>39</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>0.979933784936098</v>
+        <v>0.979933784983005</v>
       </c>
       <c r="P5" s="6" t="s">
         <v>40</v>
       </c>
       <c r="Q5" s="7" t="n">
-        <v>0.993151664730949</v>
+        <v>0.993151664747609</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.999377186450455</v>
+        <v>0.999377191513583</v>
       </c>
     </row>
     <row r="6">
@@ -1397,7 +1391,7 @@
         <v>41</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.985774863204943</v>
+        <v>0.985774870351135</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>42</v>
@@ -1409,39 +1403,39 @@
         <v>42</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.964494916249486</v>
+        <v>0.964494916609992</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3" t="n">
-        <v>0.965908193462833</v>
+        <v>0.965908195186572</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.965908193462833</v>
+        <v>0.965908195186572</v>
       </c>
       <c r="K6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.999575040995962</v>
+        <v>0.999575040979855</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>0.985731547816123</v>
+        <v>0.98573154785688</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>39</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>0.979933784936098</v>
+        <v>0.979933784983005</v>
       </c>
       <c r="P6" s="8" t="s">
         <v>39</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.993151664730949</v>
+        <v>0.993151664747609</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>0.975143582358146</v>
+        <v>0.975143586159218</v>
       </c>
     </row>
     <row r="7">
@@ -1449,7 +1443,7 @@
         <v>43</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.984219619129365</v>
+        <v>0.984219621422622</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>44</v>
@@ -1461,39 +1455,39 @@
         <v>44</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.974439597022551</v>
+        <v>0.974439597175431</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3" t="n">
-        <v>0.98546887561434</v>
+        <v>0.985468874889204</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.98546887561434</v>
+        <v>0.985468874889204</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>0.999575040995962</v>
+        <v>0.999575040979855</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>0.990258473144984</v>
+        <v>0.990258473181808</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>39</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>0.979933784936098</v>
+        <v>0.979933784983005</v>
       </c>
       <c r="P7" s="8" t="s">
         <v>39</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>0.993151664730949</v>
+        <v>0.993151664747609</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0.987195807121721</v>
+        <v>0.987195802057843</v>
       </c>
     </row>
     <row r="8">
@@ -1501,7 +1495,7 @@
         <v>45</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.951485153830059</v>
+        <v>0.951485193101285</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>46</v>
@@ -1513,39 +1507,39 @@
         <v>48</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.973836073095472</v>
+        <v>0.973836073710126</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3" t="n">
-        <v>0.939627373336213</v>
+        <v>0.939627381129929</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.804482903759715</v>
+        <v>0.804482923433398</v>
       </c>
       <c r="K8" s="6" t="s">
         <v>49</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>0.997300319860517</v>
+        <v>0.99730031971518</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>0.847828402800451</v>
+        <v>0.847828401852881</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>50</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>0.985685429503426</v>
+        <v>0.985685429734637</v>
       </c>
       <c r="P8" s="6" t="s">
         <v>51</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>0.940287785159075</v>
+        <v>0.940287785333133</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.945396131140755</v>
+        <v>0.945396127962461</v>
       </c>
     </row>
     <row r="9">
@@ -1553,7 +1547,7 @@
         <v>52</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.996989110119111</v>
+        <v>0.996989105749797</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>53</v>
@@ -1565,43 +1559,43 @@
         <v>47</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.995211832270212</v>
+        <v>0.995211832210858</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.952660131778202</v>
+        <v>0.952660131921794</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.992475624937649</v>
+        <v>0.992475622206605</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.98366871012917</v>
+        <v>0.983668706984745</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>49</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>0.997300319860517</v>
+        <v>0.99730031971518</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>0.997112251828433</v>
+        <v>0.997112251466011</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>50</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>0.985685429503426</v>
+        <v>0.985685429734637</v>
       </c>
       <c r="P9" s="8" t="s">
         <v>50</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>0.940287785159075</v>
+        <v>0.940287785333133</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0.995424708706045</v>
+        <v>0.995424681755624</v>
       </c>
     </row>
     <row r="10">
@@ -1609,7 +1603,7 @@
         <v>55</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.995469513052381</v>
+        <v>0.995469500627484</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>56</v>
@@ -1621,35 +1615,35 @@
         <v>57</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.984487609245987</v>
+        <v>0.984487609190074</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.982035840377093</v>
+        <v>0.982035840349706</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.951369988233329</v>
+        <v>0.951369987522172</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.944193811816217</v>
+        <v>0.944193811511174</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>59</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.985571290231238</v>
+        <v>0.985571289594258</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.976229904899563</v>
+        <v>0.97622990469754</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="3"/>
       <c r="P10" s="2"/>
       <c r="Q10" s="3"/>
       <c r="R10" s="3" t="n">
-        <v>0.930675294514924</v>
+        <v>0.930675282206055</v>
       </c>
     </row>
     <row r="11">
@@ -1657,7 +1651,7 @@
         <v>60</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.998300408496317</v>
+        <v>0.998300405557043</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>61</v>
@@ -1669,39 +1663,39 @@
         <v>61</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.99077239403383</v>
+        <v>0.990772393970387</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>63</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.948827781549115</v>
+        <v>0.948827781072061</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.971762010175488</v>
+        <v>0.971762017147498</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.971762010175488</v>
+        <v>0.971762017147498</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>64</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>0.994799526477391</v>
+        <v>0.994799526803795</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>0.991027893423615</v>
+        <v>0.991027892724201</v>
       </c>
       <c r="N11" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>0.908667984436548</v>
+        <v>0.908667980209571</v>
       </c>
       <c r="P11" s="6"/>
       <c r="Q11" s="7"/>
       <c r="R11" s="3" t="n">
-        <v>0.997684298092557</v>
+        <v>0.997684254462688</v>
       </c>
     </row>
     <row r="12">
@@ -1709,7 +1703,7 @@
         <v>66</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.995334597849054</v>
+        <v>0.995334578633942</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>67</v>
@@ -1721,35 +1715,35 @@
         <v>67</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.982577764855043</v>
+        <v>0.982577764655484</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3" t="n">
-        <v>0.944499430908083</v>
+        <v>0.944499434339349</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.944499430908083</v>
+        <v>0.944499434339349</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>64</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>0.994799526477391</v>
+        <v>0.994799526803795</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>0.711038761231236</v>
+        <v>0.711038758593801</v>
       </c>
       <c r="N12" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>0.908667984436548</v>
+        <v>0.908667980209571</v>
       </c>
       <c r="P12" s="6"/>
       <c r="Q12" s="7"/>
       <c r="R12" s="3" t="n">
-        <v>0.771635129733512</v>
+        <v>0.771635159550315</v>
       </c>
     </row>
     <row r="13">
@@ -1757,7 +1751,7 @@
         <v>68</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.957464756373615</v>
+        <v>0.957464770264216</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>69</v>
@@ -1769,35 +1763,35 @@
         <v>70</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.934392717811593</v>
+        <v>0.93439271726825</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="n">
-        <v>0.907751106430914</v>
+        <v>0.907751105617293</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.847252237949434</v>
+        <v>0.84725225548544</v>
       </c>
       <c r="K13" s="6" t="s">
         <v>64</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>0.994799526477391</v>
+        <v>0.994799526803795</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>0.542517905062245</v>
+        <v>0.542517903266835</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>0.908667984436548</v>
+        <v>0.908667980209571</v>
       </c>
       <c r="P13" s="6"/>
       <c r="Q13" s="7"/>
       <c r="R13" s="3" t="n">
-        <v>0.841022969900306</v>
+        <v>0.841022924443607</v>
       </c>
     </row>
     <row r="14">
@@ -1805,7 +1799,7 @@
         <v>71</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.998146874520311</v>
+        <v>0.998146875730815</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>72</v>
@@ -1817,43 +1811,43 @@
         <v>73</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.994938158549685</v>
+        <v>0.994938158413937</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>74</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.974493620999996</v>
+        <v>0.974493621233503</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.993925180554546</v>
+        <v>0.993925182660969</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.991460194711972</v>
+        <v>0.991460196151448</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>75</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.995324626236781</v>
+        <v>0.995324627330793</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.992535120953994</v>
+        <v>0.992535120940806</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>76</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.957398848117212</v>
+        <v>0.957398847892384</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>76</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>0.915585976377244</v>
+        <v>0.915585975794971</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>0.997774149994904</v>
+        <v>0.997774146210373</v>
       </c>
     </row>
     <row r="15">
@@ -1861,7 +1855,7 @@
         <v>77</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0.997720161516685</v>
+        <v>0.997720158832099</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>78</v>
@@ -1873,39 +1867,39 @@
         <v>78</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.996684575409509</v>
+        <v>0.996684575925649</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>80</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.979743628092745</v>
+        <v>0.979743627798565</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0.995235008498556</v>
+        <v>0.995235009006846</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.995235008498556</v>
+        <v>0.995235009006846</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>81</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0.480808627014228</v>
+        <v>0.480808626961847</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.830630961919803</v>
+        <v>0.830630962248236</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>82</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.954696316779994</v>
+        <v>0.954696316920534</v>
       </c>
       <c r="P15" s="2"/>
       <c r="Q15" s="3"/>
       <c r="R15" s="3" t="n">
-        <v>0.124136591318613</v>
+        <v>0.124136543010535</v>
       </c>
     </row>
     <row r="16">
@@ -1913,7 +1907,7 @@
         <v>83</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.994244367584137</v>
+        <v>0.994244385580007</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>84</v>
@@ -1925,43 +1919,43 @@
         <v>84</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.991418420361293</v>
+        <v>0.991418420322135</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>85</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.981178677303978</v>
+        <v>0.981178677269259</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.997890073647472</v>
+        <v>0.997890073511085</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.997890073647472</v>
+        <v>0.997890073511085</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>86</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.970244652019643</v>
+        <v>0.970244651996843</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.970244652019643</v>
+        <v>0.970244651996843</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>87</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.988370367422066</v>
+        <v>0.988370367437676</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.968325984027352</v>
+        <v>0.968325983966513</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.979247445962174</v>
+        <v>0.979247442874449</v>
       </c>
     </row>
     <row r="17">
@@ -1969,7 +1963,7 @@
         <v>88</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0.999233924465169</v>
+        <v>0.999233941698574</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>89</v>
@@ -1981,35 +1975,35 @@
         <v>90</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.925869318345882</v>
+        <v>0.925869317999378</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>91</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.916987691583686</v>
+        <v>0.916987691367188</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0.844528455476412</v>
+        <v>0.844528457168803</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.792129011416151</v>
+        <v>0.792128989535243</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>92</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>0.948672768843191</v>
+        <v>0.948672769079141</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.948672768843191</v>
+        <v>0.948672769079141</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="3"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="3"/>
       <c r="R17" s="3" t="n">
-        <v>0.998318979193059</v>
+        <v>0.998318975164725</v>
       </c>
     </row>
     <row r="18">
@@ -2017,7 +2011,7 @@
         <v>93</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0.956900109132159</v>
+        <v>0.956900113069297</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>94</v>
@@ -2029,24 +2023,24 @@
         <v>94</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.845720420740311</v>
+        <v>0.845720421013182</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="n">
-        <v>0.796363389036035</v>
+        <v>0.796363383376025</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.796363389036035</v>
+        <v>0.796363383376025</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>95</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>0.752297831081127</v>
+        <v>0.7522978302083</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>0.752297831081127</v>
+        <v>0.7522978302083</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="3"/>
@@ -2054,10 +2048,10 @@
         <v>96</v>
       </c>
       <c r="Q18" s="3" t="n">
-        <v>0.901574092984453</v>
+        <v>0.901574093270865</v>
       </c>
       <c r="R18" s="3" t="n">
-        <v>0.969905663618236</v>
+        <v>0.969905666335663</v>
       </c>
     </row>
     <row r="19">
@@ -2065,7 +2059,7 @@
         <v>97</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0.999980561635366</v>
+        <v>0.999980561669705</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>98</v>
@@ -2077,39 +2071,39 @@
         <v>98</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0.999995230749744</v>
+        <v>0.999995230749492</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="n">
-        <v>0.999851336466042</v>
+        <v>0.999851336491643</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.999851336466042</v>
+        <v>0.999851336491643</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>99</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>0.998961052288015</v>
+        <v>0.998961052298812</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.998961052288015</v>
+        <v>0.998961052298812</v>
       </c>
       <c r="N19" s="2" t="s">
         <v>100</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.967441621021888</v>
+        <v>0.967441621418407</v>
       </c>
       <c r="P19" s="2" t="s">
         <v>101</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>0.997513023097306</v>
+        <v>0.997513023161577</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>0.999408423329615</v>
+        <v>0.999408423516725</v>
       </c>
     </row>
     <row r="20">
@@ -2117,7 +2111,7 @@
         <v>102</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.990839008275248</v>
+        <v>0.990839010473006</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>103</v>
@@ -2129,39 +2123,39 @@
         <v>103</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.970118693520178</v>
+        <v>0.970118693726864</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3" t="n">
-        <v>0.947101462963348</v>
+        <v>0.947101463255207</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.947101462963348</v>
+        <v>0.947101463255207</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>105</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.957725007713369</v>
+        <v>0.957725008345408</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.740722621050451</v>
+        <v>0.740722621263675</v>
       </c>
       <c r="N20" s="2" t="s">
         <v>106</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.928338601031412</v>
+        <v>0.928338601315771</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>106</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>0.936826633607344</v>
+        <v>0.936826633707368</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.883182604496042</v>
+        <v>0.883182614648841</v>
       </c>
     </row>
     <row r="21">
@@ -2169,7 +2163,7 @@
         <v>107</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.996183366092605</v>
+        <v>0.996183376620369</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>108</v>
@@ -2181,43 +2175,43 @@
         <v>109</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.990794529270798</v>
+        <v>0.990794528992823</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>110</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.98860905348304</v>
+        <v>0.988609053466361</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.995274203111051</v>
+        <v>0.995274202264568</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.98197936808871</v>
+        <v>0.981979368768061</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>111</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>0.991277552948159</v>
+        <v>0.991277552763297</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>0.989949786954795</v>
+        <v>0.989949787179752</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>112</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>0.958027843030213</v>
+        <v>0.958027843028613</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>112</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>0.958027842856697</v>
+        <v>0.958027842855097</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>0.995953612024326</v>
+        <v>0.995953607248316</v>
       </c>
     </row>
     <row r="22">
@@ -2225,7 +2219,7 @@
         <v>113</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.988147728174671</v>
+        <v>0.988147727632474</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>114</v>
@@ -2237,43 +2231,43 @@
         <v>115</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0.994521225549591</v>
+        <v>0.994521225326853</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>116</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.983091970590282</v>
+        <v>0.983091970341539</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0.983947390156569</v>
+        <v>0.983947390916094</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>0.977530389103557</v>
+        <v>0.977530389706925</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>0.99651862160547</v>
+        <v>0.996518621641004</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.99651862160547</v>
+        <v>0.996518621641004</v>
       </c>
       <c r="N22" s="2" t="s">
         <v>118</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>0.932088000143203</v>
+        <v>0.932088000251616</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>118</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.958381270941474</v>
+        <v>0.95838127103415</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.985527676131329</v>
+        <v>0.985527681347115</v>
       </c>
     </row>
     <row r="23">
@@ -2281,7 +2275,7 @@
         <v>119</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.999977796574874</v>
+        <v>0.999977796576728</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>120</v>
@@ -2293,35 +2287,35 @@
         <v>120</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0.997152554254249</v>
+        <v>0.997152554293266</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3" t="n">
-        <v>0.99471604325606</v>
+        <v>0.994716043533508</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>0.99471604325606</v>
+        <v>0.994716043533508</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>121</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>0.998116134659162</v>
+        <v>0.99811613478244</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.998116134659162</v>
+        <v>0.99811613478244</v>
       </c>
       <c r="N23" s="2" t="s">
         <v>122</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>0.992624379767039</v>
+        <v>0.992624380002896</v>
       </c>
       <c r="P23" s="2"/>
       <c r="Q23" s="3"/>
       <c r="R23" s="3" t="n">
-        <v>0.99998950928761</v>
+        <v>0.999989509286429</v>
       </c>
     </row>
     <row r="24">
@@ -2377,7 +2371,7 @@
         <v>127</v>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0.9999701532808</v>
+        <v>0.999970153131709</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>128</v>
@@ -2389,35 +2383,35 @@
         <v>128</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0.999914468437142</v>
+        <v>0.999914468410852</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3" t="n">
-        <v>0.999835057995513</v>
+        <v>0.999835057913585</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.999835057995513</v>
+        <v>0.999835057913585</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>129</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>0.996899575153152</v>
+        <v>0.996899575066974</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>0.996899575153152</v>
+        <v>0.996899575066974</v>
       </c>
       <c r="N25" s="2" t="s">
         <v>130</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>0.914053274268444</v>
+        <v>0.914053275282465</v>
       </c>
       <c r="P25" s="2"/>
       <c r="Q25" s="3"/>
       <c r="R25" s="3" t="n">
-        <v>0.997931218812211</v>
+        <v>0.997931215626356</v>
       </c>
     </row>
     <row r="26">
@@ -2425,7 +2419,7 @@
         <v>131</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.999368087482014</v>
+        <v>0.999368075167037</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>132</v>
@@ -2437,43 +2431,43 @@
         <v>132</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.995835062853617</v>
+        <v>0.995835062831407</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>133</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.995865147542038</v>
+        <v>0.995865147469362</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0.986804557824535</v>
+        <v>0.986804557901822</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.986804557824535</v>
+        <v>0.986804557901822</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>134</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>0.985825843839382</v>
+        <v>0.985825843801974</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>0.985825843839382</v>
+        <v>0.985825843801974</v>
       </c>
       <c r="N26" s="2" t="s">
         <v>135</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>0.977804138512642</v>
+        <v>0.977804138460216</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>135</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>0.908745880262362</v>
+        <v>0.908745879538509</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>0.998820438844383</v>
+        <v>0.998820428122261</v>
       </c>
     </row>
     <row r="27">
@@ -2481,7 +2475,7 @@
         <v>136</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0.991323931809998</v>
+        <v>0.991323935580266</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>137</v>
@@ -2493,31 +2487,31 @@
         <v>139</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0.949421223719236</v>
+        <v>0.949421224357304</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3" t="n">
-        <v>0.875144414093871</v>
+        <v>0.875144430541776</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>0.842103236395361</v>
+        <v>0.842103252239385</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>140</v>
       </c>
       <c r="L27" s="7" t="n">
-        <v>0.989493745287417</v>
+        <v>0.989493745149078</v>
       </c>
       <c r="M27" s="7" t="n">
-        <v>0.54831345887048</v>
+        <v>0.548313458599701</v>
       </c>
       <c r="N27" s="6"/>
       <c r="O27" s="7"/>
       <c r="P27" s="6"/>
       <c r="Q27" s="7"/>
       <c r="R27" s="3" t="n">
-        <v>0.725714494601862</v>
+        <v>0.725714648921604</v>
       </c>
     </row>
     <row r="28">
@@ -2525,7 +2519,7 @@
         <v>141</v>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0.994265744437547</v>
+        <v>0.994265742578395</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>142</v>
@@ -2537,31 +2531,31 @@
         <v>143</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0.992203974046295</v>
+        <v>0.99220397390673</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3" t="n">
-        <v>0.986756134212349</v>
+        <v>0.986756133912914</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>0.969862426621788</v>
+        <v>0.969862430870855</v>
       </c>
       <c r="K28" s="6" t="s">
         <v>140</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>0.989493745287417</v>
+        <v>0.989493745149078</v>
       </c>
       <c r="M28" s="7" t="n">
-        <v>0.985557763846102</v>
+        <v>0.985557763849835</v>
       </c>
       <c r="N28" s="6"/>
       <c r="O28" s="7"/>
       <c r="P28" s="6"/>
       <c r="Q28" s="7"/>
       <c r="R28" s="3" t="n">
-        <v>0.998426211868732</v>
+        <v>0.998426213566647</v>
       </c>
     </row>
     <row r="29">
@@ -2569,463 +2563,463 @@
         <v>144</v>
       </c>
       <c r="B29" s="3" t="n">
-        <v>0.914042638364057</v>
+        <v>0.994537961750642</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>145</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>0.826204117287774</v>
+        <v>0.96057484601985</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3" t="n">
-        <v>0.797751334310876</v>
+        <v>0.926005386424851</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.531769407979438</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="L29" s="7" t="n">
-        <v>0.989493745287417</v>
-      </c>
-      <c r="M29" s="7" t="n">
-        <v>0.502264030394843</v>
-      </c>
-      <c r="N29" s="6"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="6"/>
-      <c r="Q29" s="7"/>
+        <v>0.926005386424851</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>0.966402041535507</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>0.966402041535507</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>0.988648648842376</v>
+      </c>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="3"/>
       <c r="R29" s="3" t="n">
-        <v>0.855443301955089</v>
+        <v>0.990553851536066</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B30" s="3" t="n">
-        <v>0.994537951503423</v>
+        <v>0.997211203480939</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>0.960574846051305</v>
+        <v>0.809677297640414</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3" t="n">
-        <v>0.926005384982305</v>
+        <v>0.763564608542275</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>0.926005384982305</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="L30" s="3" t="n">
-        <v>0.966402041939997</v>
-      </c>
-      <c r="M30" s="3" t="n">
-        <v>0.966402041939997</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="O30" s="3" t="n">
-        <v>0.988648649042165</v>
-      </c>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="3"/>
+        <v>0.763564608542275</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>0.822699200368759</v>
+      </c>
+      <c r="M30" s="7" t="n">
+        <v>0.433810499178233</v>
+      </c>
+      <c r="N30" s="6"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="7"/>
       <c r="R30" s="3" t="n">
-        <v>0.990553845591206</v>
+        <v>0.959733399332901</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0.979201595130134</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0.936066840683912</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0.965031393233845</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0.94202084114112</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0.94202084114112</v>
+      </c>
+      <c r="K31" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="3" t="n">
-        <v>0.997211211367285</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>0.809677297354619</v>
-      </c>
-      <c r="G31" s="2"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3" t="n">
-        <v>0.763564613951013</v>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>0.763564613951013</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="L31" s="7" t="n">
-        <v>0.822699200845167</v>
+        <v>0.822699200368759</v>
       </c>
       <c r="M31" s="7" t="n">
-        <v>0.433810499900094</v>
+        <v>0.822699200368759</v>
       </c>
       <c r="N31" s="6"/>
       <c r="O31" s="7"/>
       <c r="P31" s="6"/>
       <c r="Q31" s="7"/>
       <c r="R31" s="3" t="n">
-        <v>0.959733407276896</v>
+        <v>0.89541499698146</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.99194648722922</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B32" s="3" t="n">
-        <v>0.979201582661447</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="D32" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0.936066841399292</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="H32" s="3" t="n">
-        <v>0.965031393647406</v>
-      </c>
+        <v>0.987166551716017</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="3"/>
       <c r="I32" s="3" t="n">
-        <v>0.942020841668772</v>
+        <v>0.971914957765226</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>0.942020841668772</v>
-      </c>
-      <c r="K32" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="L32" s="7" t="n">
-        <v>0.822699200845167</v>
-      </c>
-      <c r="M32" s="7" t="n">
-        <v>0.822699200845167</v>
-      </c>
-      <c r="N32" s="6"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="6"/>
-      <c r="Q32" s="7"/>
+        <v>0.971914957765226</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>0.983005770991429</v>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>0.965867187929797</v>
+      </c>
+      <c r="N32" s="2"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="2"/>
+      <c r="Q32" s="3"/>
       <c r="R32" s="3" t="n">
-        <v>0.895414993154444</v>
+        <v>0.98168503205448</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B33" s="3" t="n">
-        <v>0.991946464271282</v>
+        <v>0.996791829147154</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>159</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0.987166551488096</v>
-      </c>
-      <c r="G33" s="2"/>
-      <c r="H33" s="3"/>
+        <v>0.971347929011293</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0.926779793958945</v>
+      </c>
       <c r="I33" s="3" t="n">
-        <v>0.971914959592856</v>
+        <v>0.958339841141185</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>0.971914959592856</v>
+        <v>0.958339841141185</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>0.983005770605164</v>
+        <v>0.8267456708621</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>0.965867188155843</v>
+        <v>0.8267456708621</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="3"/>
       <c r="P33" s="2"/>
       <c r="Q33" s="3"/>
       <c r="R33" s="3" t="n">
-        <v>0.981685023255263</v>
+        <v>0.887763751108794</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>0.996791829608519</v>
+        <v>0.974631938233094</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>0.971347929143106</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>0.92677979381067</v>
+        <v>0.987890980723224</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0.925648389418738</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>0.958339841652829</v>
+        <v>0.999743108498999</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>0.958339841652829</v>
+        <v>0.958707590298968</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>0.826745670634646</v>
+        <v>0.43129577199813</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>0.826745670634646</v>
+        <v>0.160797754767737</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="3"/>
       <c r="P34" s="2"/>
       <c r="Q34" s="3"/>
       <c r="R34" s="3" t="n">
-        <v>0.88776388540597</v>
+        <v>0.16322461962307</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0.974631943814364</v>
+        <v>0.987889323713514</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0.98789098096416</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="H35" s="3" t="n">
-        <v>0.925648389884552</v>
-      </c>
+        <v>0.977612988537665</v>
+      </c>
+      <c r="G35" s="2"/>
+      <c r="H35" s="3"/>
       <c r="I35" s="3" t="n">
-        <v>0.999743108117304</v>
+        <v>0.937108255191131</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>0.958707592156772</v>
+        <v>0.937108255191131</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>0.431295771654927</v>
+        <v>0.898847174806932</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>0.160797754844287</v>
+        <v>0.842869626226947</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="3"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="3" t="n">
-        <v>0.163224677420419</v>
+        <v>0.974928357663204</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>0.987889331039285</v>
+        <v>0.999335495603225</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="F36" s="3" t="n">
-        <v>0.97761298883184</v>
+        <v>0.992503948289454</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3" t="n">
-        <v>0.937108256523303</v>
+        <v>0.989916401342424</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.937108256523303</v>
+        <v>0.989916401342424</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.898847174499529</v>
+        <v>0.968303600220815</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.842869625399147</v>
+        <v>0.959248629031228</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="3"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="3"/>
+      <c r="P36" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q36" s="3" t="n">
+        <v>0.972597475309932</v>
+      </c>
       <c r="R36" s="3" t="n">
-        <v>0.974928376963719</v>
+        <v>0.992538193769718</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B37" s="3" t="n">
-        <v>0.999335497592149</v>
+        <v>0.996608992752013</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>177</v>
+        <v>98</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>0.992503948290037</v>
+        <v>0.954658409557154</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3" t="n">
-        <v>0.989916400630042</v>
+        <v>0.89551888167525</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.989916400630042</v>
+        <v>0.89551888167525</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>0.968303600199824</v>
+        <v>0.732165023258778</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>0.95924862884012</v>
+        <v>0.656908688833949</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="3"/>
       <c r="P37" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>0.972597475832869</v>
+        <v>0.946706660165817</v>
       </c>
       <c r="R37" s="3" t="n">
-        <v>0.992538193196534</v>
+        <v>0.94084977441347</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>0.996609000779965</v>
+        <v>0.953973633789916</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>98</v>
+        <v>182</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>0.954658409385147</v>
+        <v>0.820571179664792</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3" t="n">
-        <v>0.895518879742724</v>
+        <v>0.691459114338858</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>0.895518879742724</v>
+        <v>0.691459114338858</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>0.732165024027759</v>
+        <v>0.814121696364027</v>
       </c>
       <c r="M38" s="3" t="n">
-        <v>0.656908689233613</v>
+        <v>0.814121696364027</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="3"/>
-      <c r="P38" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="Q38" s="3" t="n">
-        <v>0.946706660713885</v>
-      </c>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="3"/>
       <c r="R38" s="3" t="n">
-        <v>0.940849790973729</v>
+        <v>0.819606280058325</v>
       </c>
     </row>
     <row r="39">
@@ -3033,7 +3027,7 @@
         <v>184</v>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0.953973626393374</v>
+        <v>0.999052672382287</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>185</v>
@@ -3045,369 +3039,325 @@
         <v>185</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0.820571179855277</v>
+        <v>0.999773004244467</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3" t="n">
-        <v>0.691459114038687</v>
+        <v>0.997679043720841</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>0.691459114038687</v>
+        <v>0.997679043720841</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>186</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>0.814121696361617</v>
+        <v>0.967598279828617</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>0.814121696361617</v>
+        <v>0.967598279828617</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="3"/>
-      <c r="P39" s="2"/>
-      <c r="Q39" s="3"/>
+      <c r="P39" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q39" s="3" t="n">
+        <v>0.932320882916883</v>
+      </c>
       <c r="R39" s="3" t="n">
-        <v>0.819606277788974</v>
+        <v>0.988716069950056</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>0.99905266647622</v>
+        <v>0.975340833576648</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0.99977300427146</v>
+        <v>0.562821812507071</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3" t="n">
-        <v>0.997679042336974</v>
+        <v>0.416003872216118</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>0.997679042336974</v>
+        <v>0.416003872216118</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>0.967598279961637</v>
+        <v>0.734845765076471</v>
       </c>
       <c r="M40" s="3" t="n">
-        <v>0.967598279961637</v>
+        <v>0.728836880498693</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="3"/>
-      <c r="P40" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q40" s="3" t="n">
-        <v>0.932320876680087</v>
-      </c>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="3"/>
       <c r="R40" s="3" t="n">
-        <v>0.988716006195344</v>
+        <v>0.817490485693601</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0.975340835478923</v>
+        <v>0.996358416382452</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.717737931500204</v>
-      </c>
-      <c r="G41" s="2"/>
-      <c r="H41" s="3"/>
+        <v>0.857208955241132</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0.910682892985077</v>
+      </c>
       <c r="I41" s="3" t="n">
-        <v>0.740483106030332</v>
+        <v>0.857836027319622</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>0.740483106030332</v>
+        <v>0.857836027319622</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>0.73484576506459</v>
+        <v>0.567227495964193</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>0.73484576506459</v>
+        <v>0.270321860444124</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="3"/>
-      <c r="P41" s="2"/>
-      <c r="Q41" s="3"/>
+      <c r="P41" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q41" s="3" t="n">
+        <v>0.981466622789426</v>
+      </c>
       <c r="R41" s="3" t="n">
-        <v>0.817490469929235</v>
+        <v>0.498953665001654</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B42" s="3" t="n">
-        <v>0.996358428040646</v>
+        <v>0.998096982715492</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>0.857208955423799</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="H42" s="3" t="n">
-        <v>0.910682893126815</v>
-      </c>
+        <v>0.965794892166284</v>
+      </c>
+      <c r="G42" s="2"/>
+      <c r="H42" s="3"/>
       <c r="I42" s="3" t="n">
-        <v>0.857836026177924</v>
+        <v>0.940623718769858</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>0.857836026177924</v>
+        <v>0.940623718769858</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>0.567227490814057</v>
+        <v>0.586961074990721</v>
       </c>
       <c r="M42" s="3" t="n">
-        <v>0.270321860201427</v>
+        <v>0.275022162781089</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="3"/>
-      <c r="P42" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q42" s="3" t="n">
-        <v>0.981466622733605</v>
-      </c>
+      <c r="P42" s="2"/>
+      <c r="Q42" s="3"/>
       <c r="R42" s="3" t="n">
-        <v>0.498953686681538</v>
+        <v>0.491571139822373</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B43" s="3" t="n">
-        <v>0.998096980390783</v>
+        <v>0.994235733371401</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>202</v>
+        <v>89</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.965794892044298</v>
+        <v>0.999915018165147</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3" t="n">
-        <v>0.940623718327597</v>
+        <v>0.994583527577986</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.940623718327597</v>
+        <v>0.994583527577986</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.58696107449826</v>
+        <v>0.719554192924328</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>0.275022162638091</v>
+        <v>0.718656820345904</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="3"/>
       <c r="P43" s="2"/>
       <c r="Q43" s="3"/>
       <c r="R43" s="3" t="n">
-        <v>0.491570915468926</v>
+        <v>0.788182679468067</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B44" s="3" t="n">
-        <v>0.994235749511032</v>
+        <v>0.989972334808116</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>89</v>
+        <v>207</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.999915018177657</v>
-      </c>
-      <c r="G44" s="2"/>
-      <c r="H44" s="3"/>
+        <v>0.984044585119664</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>0.922936621639725</v>
+      </c>
       <c r="I44" s="3" t="n">
-        <v>0.994583527351464</v>
+        <v>0.952243640465706</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>0.994583527351464</v>
-      </c>
-      <c r="K44" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="L44" s="3" t="n">
-        <v>0.719554188496143</v>
-      </c>
-      <c r="M44" s="3" t="n">
-        <v>0.718656819820427</v>
-      </c>
-      <c r="N44" s="2"/>
-      <c r="O44" s="3"/>
-      <c r="P44" s="2"/>
-      <c r="Q44" s="3"/>
+        <v>0.94971705179141</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="L44" s="7" t="n">
+        <v>0.999111403680095</v>
+      </c>
+      <c r="M44" s="7" t="n">
+        <v>0.953962159343098</v>
+      </c>
+      <c r="N44" s="6"/>
+      <c r="O44" s="7"/>
+      <c r="P44" s="6"/>
+      <c r="Q44" s="7"/>
       <c r="R44" s="3" t="n">
-        <v>0.788182601795223</v>
+        <v>0.98244996147901</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0.994871131154353</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B45" s="3" t="n">
-        <v>0.989972335380856</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="D45" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0.984978168725015</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0.904679325010897</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>0.967306964657898</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0.967306964657898</v>
+      </c>
+      <c r="K45" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="F45" s="3" t="n">
-        <v>0.984044585558769</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="H45" s="3" t="n">
-        <v>0.922936622532135</v>
-      </c>
-      <c r="I45" s="3" t="n">
-        <v>0.952243641343962</v>
-      </c>
-      <c r="J45" s="3" t="n">
-        <v>0.949717052461629</v>
-      </c>
-      <c r="K45" s="6" t="s">
-        <v>212</v>
-      </c>
       <c r="L45" s="7" t="n">
-        <v>0.0799102187135878</v>
+        <v>0.999111403680095</v>
       </c>
       <c r="M45" s="7" t="n">
-        <v>0.0596010478033871</v>
+        <v>0.999111403680095</v>
       </c>
       <c r="N45" s="6"/>
       <c r="O45" s="7"/>
       <c r="P45" s="6"/>
       <c r="Q45" s="7"/>
       <c r="R45" s="3" t="n">
-        <v>0.982449966334136</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B46" s="3" t="n">
-        <v>0.994871170695365</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>0.984978168635262</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H46" s="3" t="n">
-        <v>0.904679325987352</v>
-      </c>
-      <c r="I46" s="3" t="n">
-        <v>0.967306958360872</v>
-      </c>
-      <c r="J46" s="3" t="n">
-        <v>0.967306958360872</v>
-      </c>
-      <c r="K46" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="L46" s="7" t="n">
-        <v>0.0799102187135878</v>
-      </c>
-      <c r="M46" s="7" t="n">
-        <v>0.0799102187135878</v>
-      </c>
-      <c r="N46" s="6"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="6"/>
-      <c r="Q46" s="7"/>
-      <c r="R46" s="3" t="n">
-        <v>0.998239644693817</v>
+        <v>0.998239642694561</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3440,27 +3390,27 @@
     <mergeCell ref="O11:O13"/>
     <mergeCell ref="P11:P13"/>
     <mergeCell ref="Q11:Q13"/>
-    <mergeCell ref="K27:K29"/>
-    <mergeCell ref="L27:L29"/>
-    <mergeCell ref="M27:M29"/>
-    <mergeCell ref="N27:N29"/>
-    <mergeCell ref="O27:O29"/>
-    <mergeCell ref="P27:P29"/>
-    <mergeCell ref="Q27:Q29"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="O31:O32"/>
-    <mergeCell ref="P31:P32"/>
-    <mergeCell ref="Q31:Q32"/>
-    <mergeCell ref="K45:K46"/>
-    <mergeCell ref="L45:L46"/>
-    <mergeCell ref="M45:M46"/>
-    <mergeCell ref="N45:N46"/>
-    <mergeCell ref="O45:O46"/>
-    <mergeCell ref="P45:P46"/>
-    <mergeCell ref="Q45:Q46"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="P27:P28"/>
+    <mergeCell ref="Q27:Q28"/>
+    <mergeCell ref="K30:K31"/>
+    <mergeCell ref="L30:L31"/>
+    <mergeCell ref="M30:M31"/>
+    <mergeCell ref="N30:N31"/>
+    <mergeCell ref="O30:O31"/>
+    <mergeCell ref="P30:P31"/>
+    <mergeCell ref="Q30:Q31"/>
+    <mergeCell ref="K44:K45"/>
+    <mergeCell ref="L44:L45"/>
+    <mergeCell ref="M44:M45"/>
+    <mergeCell ref="N44:N45"/>
+    <mergeCell ref="O44:O45"/>
+    <mergeCell ref="P44:P45"/>
+    <mergeCell ref="Q44:Q45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>